<commit_message>
Fix photo links: remove spaces from Yandex Disk path
</commit_message>
<xml_diff>
--- a/kpp.xlsx
+++ b/kpp.xlsx
@@ -1731,7 +1731,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/01_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/01.jpg|yandex_disk://коробки передач на авито/01_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/02.jpg|yandex_disk://коробки передач на авито/01_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/03.jpg|yandex_disk://коробки передач на авито/01_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/01_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/01.jpg|yandex_disk://kpp_photos/01_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/02.jpg|yandex_disk://kpp_photos/01_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/03.jpg|yandex_disk://kpp_photos/01_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/04.jpg</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -1821,7 +1821,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/02_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/01.jpg|yandex_disk://коробки передач на авито/02_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/02.jpg|yandex_disk://коробки передач на авито/02_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/03.jpg|yandex_disk://коробки передач на авито/02_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/02_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/01.jpg|yandex_disk://kpp_photos/02_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/02.jpg|yandex_disk://kpp_photos/02_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/03.jpg|yandex_disk://kpp_photos/02_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/04.jpg</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/03_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/01.jpg|yandex_disk://коробки передач на авито/03_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/02.jpg|yandex_disk://коробки передач на авито/03_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/03.jpg|yandex_disk://коробки передач на авито/03_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/03_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/01.jpg|yandex_disk://kpp_photos/03_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/02.jpg|yandex_disk://kpp_photos/03_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/03.jpg|yandex_disk://kpp_photos/03_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/04.jpg</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/04_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/01.jpg|yandex_disk://коробки передач на авито/04_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/02.jpg|yandex_disk://коробки передач на авито/04_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/03.jpg|yandex_disk://коробки передач на авито/04_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/04_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/01.jpg|yandex_disk://kpp_photos/04_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/02.jpg|yandex_disk://kpp_photos/04_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/03.jpg|yandex_disk://kpp_photos/04_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/04.jpg</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/05_avtomaticheskaya_kpp_kia_sportage_ql/photos/01.jpg|yandex_disk://коробки передач на авито/05_avtomaticheskaya_kpp_kia_sportage_ql/photos/02.jpg|yandex_disk://коробки передач на авито/05_avtomaticheskaya_kpp_kia_sportage_ql/photos/03.jpg|yandex_disk://коробки передач на авито/05_avtomaticheskaya_kpp_kia_sportage_ql/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/05_avtomaticheskaya_kpp_kia_sportage_ql/photos/01.jpg|yandex_disk://kpp_photos/05_avtomaticheskaya_kpp_kia_sportage_ql/photos/02.jpg|yandex_disk://kpp_photos/05_avtomaticheskaya_kpp_kia_sportage_ql/photos/03.jpg|yandex_disk://kpp_photos/05_avtomaticheskaya_kpp_kia_sportage_ql/photos/04.jpg</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/06_avtomaticheskaya_kpp_kia_soul_ps/photos/01.jpg|yandex_disk://коробки передач на авито/06_avtomaticheskaya_kpp_kia_soul_ps/photos/02.jpg|yandex_disk://коробки передач на авито/06_avtomaticheskaya_kpp_kia_soul_ps/photos/03.jpg|yandex_disk://коробки передач на авито/06_avtomaticheskaya_kpp_kia_soul_ps/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/06_avtomaticheskaya_kpp_kia_soul_ps/photos/01.jpg|yandex_disk://kpp_photos/06_avtomaticheskaya_kpp_kia_soul_ps/photos/02.jpg|yandex_disk://kpp_photos/06_avtomaticheskaya_kpp_kia_soul_ps/photos/03.jpg|yandex_disk://kpp_photos/06_avtomaticheskaya_kpp_kia_soul_ps/photos/04.jpg</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/07_avtomaticheskaya_kpp_hyundai_i20_pb/photos/01.jpg|yandex_disk://коробки передач на авито/07_avtomaticheskaya_kpp_hyundai_i20_pb/photos/02.jpg|yandex_disk://коробки передач на авито/07_avtomaticheskaya_kpp_hyundai_i20_pb/photos/03.jpg|yandex_disk://коробки передач на авито/07_avtomaticheskaya_kpp_hyundai_i20_pb/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/07_avtomaticheskaya_kpp_hyundai_i20_pb/photos/01.jpg|yandex_disk://kpp_photos/07_avtomaticheskaya_kpp_hyundai_i20_pb/photos/02.jpg|yandex_disk://kpp_photos/07_avtomaticheskaya_kpp_hyundai_i20_pb/photos/03.jpg|yandex_disk://kpp_photos/07_avtomaticheskaya_kpp_hyundai_i20_pb/photos/04.jpg</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/08_avtomaticheskaya_kpp_kia_sportage_sl/photos/01.jpg|yandex_disk://коробки передач на авито/08_avtomaticheskaya_kpp_kia_sportage_sl/photos/02.jpg|yandex_disk://коробки передач на авито/08_avtomaticheskaya_kpp_kia_sportage_sl/photos/03.jpg|yandex_disk://коробки передач на авито/08_avtomaticheskaya_kpp_kia_sportage_sl/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/08_avtomaticheskaya_kpp_kia_sportage_sl/photos/01.jpg|yandex_disk://kpp_photos/08_avtomaticheskaya_kpp_kia_sportage_sl/photos/02.jpg|yandex_disk://kpp_photos/08_avtomaticheskaya_kpp_kia_sportage_sl/photos/03.jpg|yandex_disk://kpp_photos/08_avtomaticheskaya_kpp_kia_sportage_sl/photos/04.jpg</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/09_avtomaticheskaya_kpp_kia_sportage_sl/photos/01.jpg|yandex_disk://коробки передач на авито/09_avtomaticheskaya_kpp_kia_sportage_sl/photos/02.jpg|yandex_disk://коробки передач на авито/09_avtomaticheskaya_kpp_kia_sportage_sl/photos/03.jpg|yandex_disk://коробки передач на авито/09_avtomaticheskaya_kpp_kia_sportage_sl/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/09_avtomaticheskaya_kpp_kia_sportage_sl/photos/01.jpg|yandex_disk://kpp_photos/09_avtomaticheskaya_kpp_kia_sportage_sl/photos/02.jpg|yandex_disk://kpp_photos/09_avtomaticheskaya_kpp_kia_sportage_sl/photos/03.jpg|yandex_disk://kpp_photos/09_avtomaticheskaya_kpp_kia_sportage_sl/photos/04.jpg</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/10_avtomaticheskaya_kpp_kia_sportage_sl/photos/01.jpg|yandex_disk://коробки передач на авито/10_avtomaticheskaya_kpp_kia_sportage_sl/photos/02.jpg|yandex_disk://коробки передач на авито/10_avtomaticheskaya_kpp_kia_sportage_sl/photos/03.jpg|yandex_disk://коробки передач на авито/10_avtomaticheskaya_kpp_kia_sportage_sl/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/10_avtomaticheskaya_kpp_kia_sportage_sl/photos/01.jpg|yandex_disk://kpp_photos/10_avtomaticheskaya_kpp_kia_sportage_sl/photos/02.jpg|yandex_disk://kpp_photos/10_avtomaticheskaya_kpp_kia_sportage_sl/photos/03.jpg|yandex_disk://kpp_photos/10_avtomaticheskaya_kpp_kia_sportage_sl/photos/04.jpg</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/11_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/01.jpg|yandex_disk://коробки передач на авито/11_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/02.jpg|yandex_disk://коробки передач на авито/11_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/03.jpg|yandex_disk://коробки передач на авито/11_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/11_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/01.jpg|yandex_disk://kpp_photos/11_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/02.jpg|yandex_disk://kpp_photos/11_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/03.jpg|yandex_disk://kpp_photos/11_avtomaticheskaya_kpp_hyundai_solaris_rb/photos/04.jpg</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/12_avtomaticheskaya_kpp_kia_optima_tf/photos/01.jpg|yandex_disk://коробки передач на авито/12_avtomaticheskaya_kpp_kia_optima_tf/photos/02.jpg|yandex_disk://коробки передач на авито/12_avtomaticheskaya_kpp_kia_optima_tf/photos/03.jpg|yandex_disk://коробки передач на авито/12_avtomaticheskaya_kpp_kia_optima_tf/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/12_avtomaticheskaya_kpp_kia_optima_tf/photos/01.jpg|yandex_disk://kpp_photos/12_avtomaticheskaya_kpp_kia_optima_tf/photos/02.jpg|yandex_disk://kpp_photos/12_avtomaticheskaya_kpp_kia_optima_tf/photos/03.jpg|yandex_disk://kpp_photos/12_avtomaticheskaya_kpp_kia_optima_tf/photos/04.jpg</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/13_avtomaticheskaya_kpp_hyundai_elantra_hd/photos/01.jpg|yandex_disk://коробки передач на авито/13_avtomaticheskaya_kpp_hyundai_elantra_hd/photos/02.jpg|yandex_disk://коробки передач на авито/13_avtomaticheskaya_kpp_hyundai_elantra_hd/photos/03.jpg|yandex_disk://коробки передач на авито/13_avtomaticheskaya_kpp_hyundai_elantra_hd/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/13_avtomaticheskaya_kpp_hyundai_elantra_hd/photos/01.jpg|yandex_disk://kpp_photos/13_avtomaticheskaya_kpp_hyundai_elantra_hd/photos/02.jpg|yandex_disk://kpp_photos/13_avtomaticheskaya_kpp_hyundai_elantra_hd/photos/03.jpg|yandex_disk://kpp_photos/13_avtomaticheskaya_kpp_hyundai_elantra_hd/photos/04.jpg</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/14_mehanicheskaya_kpp_hyundai_solaris_rb/photos/01.jpg|yandex_disk://коробки передач на авито/14_mehanicheskaya_kpp_hyundai_solaris_rb/photos/03.jpg|yandex_disk://коробки передач на авито/14_mehanicheskaya_kpp_hyundai_solaris_rb/photos/04.jpg|yandex_disk://коробки передач на авито/14_mehanicheskaya_kpp_hyundai_solaris_rb/photos/05.jpg</t>
+          <t>yandex_disk://kpp_photos/14_mehanicheskaya_kpp_hyundai_solaris_rb/photos/01.jpg|yandex_disk://kpp_photos/14_mehanicheskaya_kpp_hyundai_solaris_rb/photos/03.jpg|yandex_disk://kpp_photos/14_mehanicheskaya_kpp_hyundai_solaris_rb/photos/04.jpg|yandex_disk://kpp_photos/14_mehanicheskaya_kpp_hyundai_solaris_rb/photos/05.jpg</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/15_mehanicheskaya_kpp_hyundai_i30_fd/photos/01.jpg|yandex_disk://коробки передач на авито/15_mehanicheskaya_kpp_hyundai_i30_fd/photos/02.jpg|yandex_disk://коробки передач на авито/15_mehanicheskaya_kpp_hyundai_i30_fd/photos/03.jpg|yandex_disk://коробки передач на авито/15_mehanicheskaya_kpp_hyundai_i30_fd/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/15_mehanicheskaya_kpp_hyundai_i30_fd/photos/01.jpg|yandex_disk://kpp_photos/15_mehanicheskaya_kpp_hyundai_i30_fd/photos/02.jpg|yandex_disk://kpp_photos/15_mehanicheskaya_kpp_hyundai_i30_fd/photos/03.jpg|yandex_disk://kpp_photos/15_mehanicheskaya_kpp_hyundai_i30_fd/photos/04.jpg</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
@@ -3080,7 +3080,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/16_avtomaticheskaya_kpp_audi_q3_8ub/photos/01.jpg|yandex_disk://коробки передач на авито/16_avtomaticheskaya_kpp_audi_q3_8ub/photos/02.jpg|yandex_disk://коробки передач на авито/16_avtomaticheskaya_kpp_audi_q3_8ub/photos/03.jpg|yandex_disk://коробки передач на авито/16_avtomaticheskaya_kpp_audi_q3_8ub/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/16_avtomaticheskaya_kpp_audi_q3_8ub/photos/01.jpg|yandex_disk://kpp_photos/16_avtomaticheskaya_kpp_audi_q3_8ub/photos/02.jpg|yandex_disk://kpp_photos/16_avtomaticheskaya_kpp_audi_q3_8ub/photos/03.jpg|yandex_disk://kpp_photos/16_avtomaticheskaya_kpp_audi_q3_8ub/photos/04.jpg</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/17_avtomaticheskaya_kpp_audi_q5_8rb/photos/01.jpg|yandex_disk://коробки передач на авито/17_avtomaticheskaya_kpp_audi_q5_8rb/photos/02.jpg|yandex_disk://коробки передач на авито/17_avtomaticheskaya_kpp_audi_q5_8rb/photos/03.jpg|yandex_disk://коробки передач на авито/17_avtomaticheskaya_kpp_audi_q5_8rb/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/17_avtomaticheskaya_kpp_audi_q5_8rb/photos/01.jpg|yandex_disk://kpp_photos/17_avtomaticheskaya_kpp_audi_q5_8rb/photos/02.jpg|yandex_disk://kpp_photos/17_avtomaticheskaya_kpp_audi_q5_8rb/photos/03.jpg|yandex_disk://kpp_photos/17_avtomaticheskaya_kpp_audi_q5_8rb/photos/04.jpg</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/18_avtomaticheskaya_kpp_audi_a4_allroad_8kh/photos/01.jpg|yandex_disk://коробки передач на авито/18_avtomaticheskaya_kpp_audi_a4_allroad_8kh/photos/02.jpg|yandex_disk://коробки передач на авито/18_avtomaticheskaya_kpp_audi_a4_allroad_8kh/photos/03.jpg|yandex_disk://коробки передач на авито/18_avtomaticheskaya_kpp_audi_a4_allroad_8kh/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/18_avtomaticheskaya_kpp_audi_a4_allroad_8kh/photos/01.jpg|yandex_disk://kpp_photos/18_avtomaticheskaya_kpp_audi_a4_allroad_8kh/photos/02.jpg|yandex_disk://kpp_photos/18_avtomaticheskaya_kpp_audi_a4_allroad_8kh/photos/03.jpg|yandex_disk://kpp_photos/18_avtomaticheskaya_kpp_audi_a4_allroad_8kh/photos/04.jpg</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/19_avtomaticheskaya_kpp_audi_a4_b8_8k2/photos/01.jpg|yandex_disk://коробки передач на авито/19_avtomaticheskaya_kpp_audi_a4_b8_8k2/photos/02.jpg|yandex_disk://коробки передач на авито/19_avtomaticheskaya_kpp_audi_a4_b8_8k2/photos/03.jpg|yandex_disk://коробки передач на авито/19_avtomaticheskaya_kpp_audi_a4_b8_8k2/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/19_avtomaticheskaya_kpp_audi_a4_b8_8k2/photos/01.jpg|yandex_disk://kpp_photos/19_avtomaticheskaya_kpp_audi_a4_b8_8k2/photos/02.jpg|yandex_disk://kpp_photos/19_avtomaticheskaya_kpp_audi_a4_b8_8k2/photos/03.jpg|yandex_disk://kpp_photos/19_avtomaticheskaya_kpp_audi_a4_b8_8k2/photos/04.jpg</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/20_avtomaticheskaya_kpp_bmw_x1_e84/photos/01.jpg|yandex_disk://коробки передач на авито/20_avtomaticheskaya_kpp_bmw_x1_e84/photos/02.jpg|yandex_disk://коробки передач на авито/20_avtomaticheskaya_kpp_bmw_x1_e84/photos/03.jpg|yandex_disk://коробки передач на авито/20_avtomaticheskaya_kpp_bmw_x1_e84/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/20_avtomaticheskaya_kpp_bmw_x1_e84/photos/01.jpg|yandex_disk://kpp_photos/20_avtomaticheskaya_kpp_bmw_x1_e84/photos/02.jpg|yandex_disk://kpp_photos/20_avtomaticheskaya_kpp_bmw_x1_e84/photos/03.jpg|yandex_disk://kpp_photos/20_avtomaticheskaya_kpp_bmw_x1_e84/photos/04.jpg</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/21_avtomaticheskaya_kpp_bmw_5_series_f07/photos/01.jpg|yandex_disk://коробки передач на авито/21_avtomaticheskaya_kpp_bmw_5_series_f07/photos/02.jpg|yandex_disk://коробки передач на авито/21_avtomaticheskaya_kpp_bmw_5_series_f07/photos/03.jpg|yandex_disk://коробки передач на авито/21_avtomaticheskaya_kpp_bmw_5_series_f07/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/21_avtomaticheskaya_kpp_bmw_5_series_f07/photos/01.jpg|yandex_disk://kpp_photos/21_avtomaticheskaya_kpp_bmw_5_series_f07/photos/02.jpg|yandex_disk://kpp_photos/21_avtomaticheskaya_kpp_bmw_5_series_f07/photos/03.jpg|yandex_disk://kpp_photos/21_avtomaticheskaya_kpp_bmw_5_series_f07/photos/04.jpg</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/22_avtomaticheskaya_kpp_bmw_5_series_e60/photos/01.jpg|yandex_disk://коробки передач на авито/22_avtomaticheskaya_kpp_bmw_5_series_e60/photos/03.jpg|yandex_disk://коробки передач на авито/22_avtomaticheskaya_kpp_bmw_5_series_e60/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/22_avtomaticheskaya_kpp_bmw_5_series_e60/photos/01.jpg|yandex_disk://kpp_photos/22_avtomaticheskaya_kpp_bmw_5_series_e60/photos/03.jpg|yandex_disk://kpp_photos/22_avtomaticheskaya_kpp_bmw_5_series_e60/photos/04.jpg</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/23_avtomaticheskaya_kpp_bmw_3_series_f30/photos/01.jpg|yandex_disk://коробки передач на авито/23_avtomaticheskaya_kpp_bmw_3_series_f30/photos/02.jpg|yandex_disk://коробки передач на авито/23_avtomaticheskaya_kpp_bmw_3_series_f30/photos/03.jpg|yandex_disk://коробки передач на авито/23_avtomaticheskaya_kpp_bmw_3_series_f30/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/23_avtomaticheskaya_kpp_bmw_3_series_f30/photos/01.jpg|yandex_disk://kpp_photos/23_avtomaticheskaya_kpp_bmw_3_series_f30/photos/02.jpg|yandex_disk://kpp_photos/23_avtomaticheskaya_kpp_bmw_3_series_f30/photos/03.jpg|yandex_disk://kpp_photos/23_avtomaticheskaya_kpp_bmw_3_series_f30/photos/04.jpg</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/24_avtomaticheskaya_kpp_bmw_5_series_e60/photos/01.jpg|yandex_disk://коробки передач на авито/24_avtomaticheskaya_kpp_bmw_5_series_e60/photos/02.jpg|yandex_disk://коробки передач на авито/24_avtomaticheskaya_kpp_bmw_5_series_e60/photos/03.jpg|yandex_disk://коробки передач на авито/24_avtomaticheskaya_kpp_bmw_5_series_e60/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/24_avtomaticheskaya_kpp_bmw_5_series_e60/photos/01.jpg|yandex_disk://kpp_photos/24_avtomaticheskaya_kpp_bmw_5_series_e60/photos/02.jpg|yandex_disk://kpp_photos/24_avtomaticheskaya_kpp_bmw_5_series_e60/photos/03.jpg|yandex_disk://kpp_photos/24_avtomaticheskaya_kpp_bmw_5_series_e60/photos/04.jpg</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/25_avtomaticheskaya_kpp_bmw_3_series_e91/photos/01.jpg|yandex_disk://коробки передач на авито/25_avtomaticheskaya_kpp_bmw_3_series_e91/photos/02.jpg|yandex_disk://коробки передач на авито/25_avtomaticheskaya_kpp_bmw_3_series_e91/photos/03.jpg|yandex_disk://коробки передач на авито/25_avtomaticheskaya_kpp_bmw_3_series_e91/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/25_avtomaticheskaya_kpp_bmw_3_series_e91/photos/01.jpg|yandex_disk://kpp_photos/25_avtomaticheskaya_kpp_bmw_3_series_e91/photos/02.jpg|yandex_disk://kpp_photos/25_avtomaticheskaya_kpp_bmw_3_series_e91/photos/03.jpg|yandex_disk://kpp_photos/25_avtomaticheskaya_kpp_bmw_3_series_e91/photos/04.jpg</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/26_avtomaticheskaya_kpp_bmw_3_series_e90/photos/01.jpg|yandex_disk://коробки передач на авито/26_avtomaticheskaya_kpp_bmw_3_series_e90/photos/02.jpg|yandex_disk://коробки передач на авито/26_avtomaticheskaya_kpp_bmw_3_series_e90/photos/03.jpg|yandex_disk://коробки передач на авито/26_avtomaticheskaya_kpp_bmw_3_series_e90/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/26_avtomaticheskaya_kpp_bmw_3_series_e90/photos/01.jpg|yandex_disk://kpp_photos/26_avtomaticheskaya_kpp_bmw_3_series_e90/photos/02.jpg|yandex_disk://kpp_photos/26_avtomaticheskaya_kpp_bmw_3_series_e90/photos/03.jpg|yandex_disk://kpp_photos/26_avtomaticheskaya_kpp_bmw_3_series_e90/photos/04.jpg</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/27_avtomaticheskaya_kpp_bmw_5_series_e60/photos/01.jpg|yandex_disk://коробки передач на авито/27_avtomaticheskaya_kpp_bmw_5_series_e60/photos/02.jpg|yandex_disk://коробки передач на авито/27_avtomaticheskaya_kpp_bmw_5_series_e60/photos/03.jpg|yandex_disk://коробки передач на авито/27_avtomaticheskaya_kpp_bmw_5_series_e60/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/27_avtomaticheskaya_kpp_bmw_5_series_e60/photos/01.jpg|yandex_disk://kpp_photos/27_avtomaticheskaya_kpp_bmw_5_series_e60/photos/02.jpg|yandex_disk://kpp_photos/27_avtomaticheskaya_kpp_bmw_5_series_e60/photos/03.jpg|yandex_disk://kpp_photos/27_avtomaticheskaya_kpp_bmw_5_series_e60/photos/04.jpg</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
@@ -4150,7 +4150,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/28_avtomaticheskaya_kpp_bmw_1_series_e87/photos/01.jpg|yandex_disk://коробки передач на авито/28_avtomaticheskaya_kpp_bmw_1_series_e87/photos/02.jpg|yandex_disk://коробки передач на авито/28_avtomaticheskaya_kpp_bmw_1_series_e87/photos/03.jpg|yandex_disk://коробки передач на авито/28_avtomaticheskaya_kpp_bmw_1_series_e87/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/28_avtomaticheskaya_kpp_bmw_1_series_e87/photos/01.jpg|yandex_disk://kpp_photos/28_avtomaticheskaya_kpp_bmw_1_series_e87/photos/02.jpg|yandex_disk://kpp_photos/28_avtomaticheskaya_kpp_bmw_1_series_e87/photos/03.jpg|yandex_disk://kpp_photos/28_avtomaticheskaya_kpp_bmw_1_series_e87/photos/04.jpg</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/29_avtomaticheskaya_kpp_bmw_1_series_e87/photos/01.jpg|yandex_disk://коробки передач на авито/29_avtomaticheskaya_kpp_bmw_1_series_e87/photos/02.jpg|yandex_disk://коробки передач на авито/29_avtomaticheskaya_kpp_bmw_1_series_e87/photos/03.jpg|yandex_disk://коробки передач на авито/29_avtomaticheskaya_kpp_bmw_1_series_e87/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/29_avtomaticheskaya_kpp_bmw_1_series_e87/photos/01.jpg|yandex_disk://kpp_photos/29_avtomaticheskaya_kpp_bmw_1_series_e87/photos/02.jpg|yandex_disk://kpp_photos/29_avtomaticheskaya_kpp_bmw_1_series_e87/photos/03.jpg|yandex_disk://kpp_photos/29_avtomaticheskaya_kpp_bmw_1_series_e87/photos/04.jpg</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/30_avtomaticheskaya_kpp_chery_tiggo_7_pro_max_t1e/photos/01.jpg|yandex_disk://коробки передач на авито/30_avtomaticheskaya_kpp_chery_tiggo_7_pro_max_t1e/photos/02.jpg|yandex_disk://коробки передач на авито/30_avtomaticheskaya_kpp_chery_tiggo_7_pro_max_t1e/photos/03.jpg|yandex_disk://коробки передач на авито/30_avtomaticheskaya_kpp_chery_tiggo_7_pro_max_t1e/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/30_avtomaticheskaya_kpp_chery_tiggo_7_pro_max_t1e/photos/01.jpg|yandex_disk://kpp_photos/30_avtomaticheskaya_kpp_chery_tiggo_7_pro_max_t1e/photos/02.jpg|yandex_disk://kpp_photos/30_avtomaticheskaya_kpp_chery_tiggo_7_pro_max_t1e/photos/03.jpg|yandex_disk://kpp_photos/30_avtomaticheskaya_kpp_chery_tiggo_7_pro_max_t1e/photos/04.jpg</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/31_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/01.jpg|yandex_disk://коробки передач на авито/31_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/02.jpg|yandex_disk://коробки передач на авито/31_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/03.jpg|yandex_disk://коробки передач на авито/31_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/31_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/01.jpg|yandex_disk://kpp_photos/31_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/02.jpg|yandex_disk://kpp_photos/31_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/03.jpg|yandex_disk://kpp_photos/31_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/04.jpg</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/32_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/01.jpg|yandex_disk://коробки передач на авито/32_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/02.jpg|yandex_disk://коробки передач на авито/32_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/03.jpg|yandex_disk://коробки передач на авито/32_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/32_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/01.jpg|yandex_disk://kpp_photos/32_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/02.jpg|yandex_disk://kpp_photos/32_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/03.jpg|yandex_disk://kpp_photos/32_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/04.jpg</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/33_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/01.jpg|yandex_disk://коробки передач на авито/33_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/02.jpg|yandex_disk://коробки передач на авито/33_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/03.jpg|yandex_disk://коробки передач на авито/33_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/33_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/01.jpg|yandex_disk://kpp_photos/33_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/02.jpg|yandex_disk://kpp_photos/33_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/03.jpg|yandex_disk://kpp_photos/33_avtomaticheskaya_kpp_chevrolet_captiva_c100/photos/04.jpg</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/34_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/01.jpg|yandex_disk://коробки передач на авито/34_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/02.jpg|yandex_disk://коробки передач на авито/34_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/03.jpg|yandex_disk://коробки передач на авито/34_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/34_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/01.jpg|yandex_disk://kpp_photos/34_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/02.jpg|yandex_disk://kpp_photos/34_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/03.jpg|yandex_disk://kpp_photos/34_avtomaticheskaya_kpp_chevrolet_aveo_t300/photos/04.jpg</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/35_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/01.jpg|yandex_disk://коробки передач на авито/35_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/02.jpg|yandex_disk://коробки передач на авито/35_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/03.jpg|yandex_disk://коробки передач на авито/35_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/35_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/01.jpg|yandex_disk://kpp_photos/35_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/02.jpg|yandex_disk://kpp_photos/35_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/03.jpg|yandex_disk://kpp_photos/35_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/04.jpg</t>
         </is>
       </c>
       <c r="X39" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/36_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/01.jpg|yandex_disk://коробки передач на авито/36_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/02.jpg|yandex_disk://коробки передач на авито/36_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/03.jpg</t>
+          <t>yandex_disk://kpp_photos/36_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/01.jpg|yandex_disk://kpp_photos/36_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/02.jpg|yandex_disk://kpp_photos/36_avtomaticheskaya_kpp_chevrolet_cruze_j300/photos/03.jpg</t>
         </is>
       </c>
       <c r="X40" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/37_avtomaticheskaya_kpp_chevrolet_captiva_c140/photos/01.jpg|yandex_disk://коробки передач на авито/37_avtomaticheskaya_kpp_chevrolet_captiva_c140/photos/02.jpg|yandex_disk://коробки передач на авито/37_avtomaticheskaya_kpp_chevrolet_captiva_c140/photos/03.jpg|yandex_disk://коробки передач на авито/37_avtomaticheskaya_kpp_chevrolet_captiva_c140/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/37_avtomaticheskaya_kpp_chevrolet_captiva_c140/photos/01.jpg|yandex_disk://kpp_photos/37_avtomaticheskaya_kpp_chevrolet_captiva_c140/photos/02.jpg|yandex_disk://kpp_photos/37_avtomaticheskaya_kpp_chevrolet_captiva_c140/photos/03.jpg|yandex_disk://kpp_photos/37_avtomaticheskaya_kpp_chevrolet_captiva_c140/photos/04.jpg</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
@@ -5044,7 +5044,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/38_mehanicheskaya_kpp_chevrolet_cruze_j300/photos/01.jpg|yandex_disk://коробки передач на авито/38_mehanicheskaya_kpp_chevrolet_cruze_j300/photos/02.jpg|yandex_disk://коробки передач на авито/38_mehanicheskaya_kpp_chevrolet_cruze_j300/photos/03.jpg|yandex_disk://коробки передач на авито/38_mehanicheskaya_kpp_chevrolet_cruze_j300/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/38_mehanicheskaya_kpp_chevrolet_cruze_j300/photos/01.jpg|yandex_disk://kpp_photos/38_mehanicheskaya_kpp_chevrolet_cruze_j300/photos/02.jpg|yandex_disk://kpp_photos/38_mehanicheskaya_kpp_chevrolet_cruze_j300/photos/03.jpg|yandex_disk://kpp_photos/38_mehanicheskaya_kpp_chevrolet_cruze_j300/photos/04.jpg</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/39_avtomaticheskaya_kpp_dodge_caliber_pm/photos/01.jpg|yandex_disk://коробки передач на авито/39_avtomaticheskaya_kpp_dodge_caliber_pm/photos/02.jpg|yandex_disk://коробки передач на авито/39_avtomaticheskaya_kpp_dodge_caliber_pm/photos/03.jpg|yandex_disk://коробки передач на авито/39_avtomaticheskaya_kpp_dodge_caliber_pm/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/39_avtomaticheskaya_kpp_dodge_caliber_pm/photos/01.jpg|yandex_disk://kpp_photos/39_avtomaticheskaya_kpp_dodge_caliber_pm/photos/02.jpg|yandex_disk://kpp_photos/39_avtomaticheskaya_kpp_dodge_caliber_pm/photos/03.jpg|yandex_disk://kpp_photos/39_avtomaticheskaya_kpp_dodge_caliber_pm/photos/04.jpg</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
@@ -5224,7 +5224,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/40_avtomaticheskaya_kpp_ford_kuga_cbs/photos/01.jpg|yandex_disk://коробки передач на авито/40_avtomaticheskaya_kpp_ford_kuga_cbs/photos/02.jpg|yandex_disk://коробки передач на авито/40_avtomaticheskaya_kpp_ford_kuga_cbs/photos/03.jpg|yandex_disk://коробки передач на авито/40_avtomaticheskaya_kpp_ford_kuga_cbs/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/40_avtomaticheskaya_kpp_ford_kuga_cbs/photos/01.jpg|yandex_disk://kpp_photos/40_avtomaticheskaya_kpp_ford_kuga_cbs/photos/02.jpg|yandex_disk://kpp_photos/40_avtomaticheskaya_kpp_ford_kuga_cbs/photos/03.jpg|yandex_disk://kpp_photos/40_avtomaticheskaya_kpp_ford_kuga_cbs/photos/04.jpg</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/41_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/01.jpg|yandex_disk://коробки передач на авито/41_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/02.jpg|yandex_disk://коробки передач на авито/41_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/03.jpg|yandex_disk://коробки передач на авито/41_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/41_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/01.jpg|yandex_disk://kpp_photos/41_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/02.jpg|yandex_disk://kpp_photos/41_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/03.jpg|yandex_disk://kpp_photos/41_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/04.jpg</t>
         </is>
       </c>
       <c r="X45" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/42_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/01.jpg|yandex_disk://коробки передач на авито/42_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/02.jpg|yandex_disk://коробки передач на авито/42_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/03.jpg|yandex_disk://коробки передач на авито/42_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/42_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/01.jpg|yandex_disk://kpp_photos/42_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/02.jpg|yandex_disk://kpp_photos/42_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/03.jpg|yandex_disk://kpp_photos/42_avtomaticheskaya_kpp_ford_focus_3_cb8/photos/04.jpg</t>
         </is>
       </c>
       <c r="X46" t="inlineStr">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/43_avtomaticheskaya_kpp_ford_mondeo_be/photos/01.jpg|yandex_disk://коробки передач на авито/43_avtomaticheskaya_kpp_ford_mondeo_be/photos/02.jpg|yandex_disk://коробки передач на авито/43_avtomaticheskaya_kpp_ford_mondeo_be/photos/03.jpg|yandex_disk://коробки передач на авито/43_avtomaticheskaya_kpp_ford_mondeo_be/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/43_avtomaticheskaya_kpp_ford_mondeo_be/photos/01.jpg|yandex_disk://kpp_photos/43_avtomaticheskaya_kpp_ford_mondeo_be/photos/02.jpg|yandex_disk://kpp_photos/43_avtomaticheskaya_kpp_ford_mondeo_be/photos/03.jpg|yandex_disk://kpp_photos/43_avtomaticheskaya_kpp_ford_mondeo_be/photos/04.jpg</t>
         </is>
       </c>
       <c r="X47" t="inlineStr">
@@ -5582,7 +5582,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/44_avtomaticheskaya_kpp_ford_fiesta_cbk/photos/01.jpg|yandex_disk://коробки передач на авито/44_avtomaticheskaya_kpp_ford_fiesta_cbk/photos/02.jpg|yandex_disk://коробки передач на авито/44_avtomaticheskaya_kpp_ford_fiesta_cbk/photos/03.jpg|yandex_disk://коробки передач на авито/44_avtomaticheskaya_kpp_ford_fiesta_cbk/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/44_avtomaticheskaya_kpp_ford_fiesta_cbk/photos/01.jpg|yandex_disk://kpp_photos/44_avtomaticheskaya_kpp_ford_fiesta_cbk/photos/02.jpg|yandex_disk://kpp_photos/44_avtomaticheskaya_kpp_ford_fiesta_cbk/photos/03.jpg|yandex_disk://kpp_photos/44_avtomaticheskaya_kpp_ford_fiesta_cbk/photos/04.jpg</t>
         </is>
       </c>
       <c r="X48" t="inlineStr">
@@ -5672,7 +5672,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/45_avtomaticheskaya_kpp_ford_mondeo_bg/photos/01.jpg|yandex_disk://коробки передач на авито/45_avtomaticheskaya_kpp_ford_mondeo_bg/photos/02.jpg|yandex_disk://коробки передач на авито/45_avtomaticheskaya_kpp_ford_mondeo_bg/photos/03.jpg|yandex_disk://коробки передач на авито/45_avtomaticheskaya_kpp_ford_mondeo_bg/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/45_avtomaticheskaya_kpp_ford_mondeo_bg/photos/01.jpg|yandex_disk://kpp_photos/45_avtomaticheskaya_kpp_ford_mondeo_bg/photos/02.jpg|yandex_disk://kpp_photos/45_avtomaticheskaya_kpp_ford_mondeo_bg/photos/03.jpg|yandex_disk://kpp_photos/45_avtomaticheskaya_kpp_ford_mondeo_bg/photos/04.jpg</t>
         </is>
       </c>
       <c r="X49" t="inlineStr">
@@ -5762,7 +5762,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/46_avtomaticheskaya_kpp_great_wall_poer_x/photos/01.jpg|yandex_disk://коробки передач на авито/46_avtomaticheskaya_kpp_great_wall_poer_x/photos/02.jpg|yandex_disk://коробки передач на авито/46_avtomaticheskaya_kpp_great_wall_poer_x/photos/03.jpg|yandex_disk://коробки передач на авито/46_avtomaticheskaya_kpp_great_wall_poer_x/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/46_avtomaticheskaya_kpp_great_wall_poer_x/photos/01.jpg|yandex_disk://kpp_photos/46_avtomaticheskaya_kpp_great_wall_poer_x/photos/02.jpg|yandex_disk://kpp_photos/46_avtomaticheskaya_kpp_great_wall_poer_x/photos/03.jpg|yandex_disk://kpp_photos/46_avtomaticheskaya_kpp_great_wall_poer_x/photos/04.jpg</t>
         </is>
       </c>
       <c r="X50" t="inlineStr">
@@ -5852,7 +5852,7 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/47_avtomaticheskaya_kpp_great_wall_poer_x/photos/01.jpg|yandex_disk://коробки передач на авито/47_avtomaticheskaya_kpp_great_wall_poer_x/photos/02.jpg|yandex_disk://коробки передач на авито/47_avtomaticheskaya_kpp_great_wall_poer_x/photos/03.jpg|yandex_disk://коробки передач на авито/47_avtomaticheskaya_kpp_great_wall_poer_x/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/47_avtomaticheskaya_kpp_great_wall_poer_x/photos/01.jpg|yandex_disk://kpp_photos/47_avtomaticheskaya_kpp_great_wall_poer_x/photos/02.jpg|yandex_disk://kpp_photos/47_avtomaticheskaya_kpp_great_wall_poer_x/photos/03.jpg|yandex_disk://kpp_photos/47_avtomaticheskaya_kpp_great_wall_poer_x/photos/04.jpg</t>
         </is>
       </c>
       <c r="X51" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/48_avtomaticheskaya_kpp_haval_h6_x/photos/01.jpg|yandex_disk://коробки передач на авито/48_avtomaticheskaya_kpp_haval_h6_x/photos/02.jpg|yandex_disk://коробки передач на авито/48_avtomaticheskaya_kpp_haval_h6_x/photos/03.jpg|yandex_disk://коробки передач на авито/48_avtomaticheskaya_kpp_haval_h6_x/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/48_avtomaticheskaya_kpp_haval_h6_x/photos/01.jpg|yandex_disk://kpp_photos/48_avtomaticheskaya_kpp_haval_h6_x/photos/02.jpg|yandex_disk://kpp_photos/48_avtomaticheskaya_kpp_haval_h6_x/photos/03.jpg|yandex_disk://kpp_photos/48_avtomaticheskaya_kpp_haval_h6_x/photos/04.jpg</t>
         </is>
       </c>
       <c r="X52" t="inlineStr">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/49_avtomaticheskaya_kpp_honda_freed_gb7/photos/01.jpg|yandex_disk://коробки передач на авито/49_avtomaticheskaya_kpp_honda_freed_gb7/photos/02.jpg|yandex_disk://коробки передач на авито/49_avtomaticheskaya_kpp_honda_freed_gb7/photos/03.jpg|yandex_disk://коробки передач на авито/49_avtomaticheskaya_kpp_honda_freed_gb7/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/49_avtomaticheskaya_kpp_honda_freed_gb7/photos/01.jpg|yandex_disk://kpp_photos/49_avtomaticheskaya_kpp_honda_freed_gb7/photos/02.jpg|yandex_disk://kpp_photos/49_avtomaticheskaya_kpp_honda_freed_gb7/photos/03.jpg|yandex_disk://kpp_photos/49_avtomaticheskaya_kpp_honda_freed_gb7/photos/04.jpg</t>
         </is>
       </c>
       <c r="X53" t="inlineStr">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/50_avtomaticheskaya_kpp_honda_cr_v_rm1/photos/01.jpg|yandex_disk://коробки передач на авито/50_avtomaticheskaya_kpp_honda_cr_v_rm1/photos/02.jpg|yandex_disk://коробки передач на авито/50_avtomaticheskaya_kpp_honda_cr_v_rm1/photos/03.jpg|yandex_disk://коробки передач на авито/50_avtomaticheskaya_kpp_honda_cr_v_rm1/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/50_avtomaticheskaya_kpp_honda_cr_v_rm1/photos/01.jpg|yandex_disk://kpp_photos/50_avtomaticheskaya_kpp_honda_cr_v_rm1/photos/02.jpg|yandex_disk://kpp_photos/50_avtomaticheskaya_kpp_honda_cr_v_rm1/photos/03.jpg|yandex_disk://kpp_photos/50_avtomaticheskaya_kpp_honda_cr_v_rm1/photos/04.jpg</t>
         </is>
       </c>
       <c r="X54" t="inlineStr">
@@ -6209,7 +6209,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/51_avtomaticheskaya_kpp_honda_cr_v_re7/photos/01.jpg|yandex_disk://коробки передач на авито/51_avtomaticheskaya_kpp_honda_cr_v_re7/photos/02.jpg|yandex_disk://коробки передач на авито/51_avtomaticheskaya_kpp_honda_cr_v_re7/photos/03.jpg|yandex_disk://коробки передач на авито/51_avtomaticheskaya_kpp_honda_cr_v_re7/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/51_avtomaticheskaya_kpp_honda_cr_v_re7/photos/01.jpg|yandex_disk://kpp_photos/51_avtomaticheskaya_kpp_honda_cr_v_re7/photos/02.jpg|yandex_disk://kpp_photos/51_avtomaticheskaya_kpp_honda_cr_v_re7/photos/03.jpg|yandex_disk://kpp_photos/51_avtomaticheskaya_kpp_honda_cr_v_re7/photos/04.jpg</t>
         </is>
       </c>
       <c r="X55" t="inlineStr">
@@ -6299,7 +6299,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/52_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/01.jpg|yandex_disk://коробки передач на авито/52_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/02.jpg|yandex_disk://коробки передач на авито/52_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/03.jpg|yandex_disk://коробки передач на авито/52_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/52_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/01.jpg|yandex_disk://kpp_photos/52_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/02.jpg|yandex_disk://kpp_photos/52_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/03.jpg|yandex_disk://kpp_photos/52_avtomaticheskaya_kpp_hyundai_ix35_lm/photos/04.jpg</t>
         </is>
       </c>
       <c r="X56" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/53_avtomaticheskaya_kpp_infiniti_fx37_s51/photos/01.jpg|yandex_disk://коробки передач на авито/53_avtomaticheskaya_kpp_infiniti_fx37_s51/photos/02.jpg|yandex_disk://коробки передач на авито/53_avtomaticheskaya_kpp_infiniti_fx37_s51/photos/03.jpg|yandex_disk://коробки передач на авито/53_avtomaticheskaya_kpp_infiniti_fx37_s51/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/53_avtomaticheskaya_kpp_infiniti_fx37_s51/photos/01.jpg|yandex_disk://kpp_photos/53_avtomaticheskaya_kpp_infiniti_fx37_s51/photos/02.jpg|yandex_disk://kpp_photos/53_avtomaticheskaya_kpp_infiniti_fx37_s51/photos/03.jpg|yandex_disk://kpp_photos/53_avtomaticheskaya_kpp_infiniti_fx37_s51/photos/04.jpg</t>
         </is>
       </c>
       <c r="X57" t="inlineStr">
@@ -6478,7 +6478,7 @@
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/54_avtomaticheskaya_kpp_land_rover_range_rover_evoque_l538/photos/01.jpg|yandex_disk://коробки передач на авито/54_avtomaticheskaya_kpp_land_rover_range_rover_evoque_l538/photos/02.jpg|yandex_disk://коробки передач на авито/54_avtomaticheskaya_kpp_land_rover_range_rover_evoque_l538/photos/03.jpg|yandex_disk://коробки передач на авито/54_avtomaticheskaya_kpp_land_rover_range_rover_evoque_l538/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/54_avtomaticheskaya_kpp_land_rover_range_rover_evoque_l538/photos/01.jpg|yandex_disk://kpp_photos/54_avtomaticheskaya_kpp_land_rover_range_rover_evoque_l538/photos/02.jpg|yandex_disk://kpp_photos/54_avtomaticheskaya_kpp_land_rover_range_rover_evoque_l538/photos/03.jpg|yandex_disk://kpp_photos/54_avtomaticheskaya_kpp_land_rover_range_rover_evoque_l538/photos/04.jpg</t>
         </is>
       </c>
       <c r="X58" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/55_avtomaticheskaya_kpp_lexus_is250_gse20/photos/01.jpg|yandex_disk://коробки передач на авито/55_avtomaticheskaya_kpp_lexus_is250_gse20/photos/02.jpg|yandex_disk://коробки передач на авито/55_avtomaticheskaya_kpp_lexus_is250_gse20/photos/03.jpg|yandex_disk://коробки передач на авито/55_avtomaticheskaya_kpp_lexus_is250_gse20/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/55_avtomaticheskaya_kpp_lexus_is250_gse20/photos/01.jpg|yandex_disk://kpp_photos/55_avtomaticheskaya_kpp_lexus_is250_gse20/photos/02.jpg|yandex_disk://kpp_photos/55_avtomaticheskaya_kpp_lexus_is250_gse20/photos/03.jpg|yandex_disk://kpp_photos/55_avtomaticheskaya_kpp_lexus_is250_gse20/photos/04.jpg</t>
         </is>
       </c>
       <c r="X59" t="inlineStr">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/56_avtomaticheskaya_kpp_lexus_rx400_mhu38/photos/01.jpg|yandex_disk://коробки передач на авито/56_avtomaticheskaya_kpp_lexus_rx400_mhu38/photos/02.jpg|yandex_disk://коробки передач на авито/56_avtomaticheskaya_kpp_lexus_rx400_mhu38/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/56_avtomaticheskaya_kpp_lexus_rx400_mhu38/photos/01.jpg|yandex_disk://kpp_photos/56_avtomaticheskaya_kpp_lexus_rx400_mhu38/photos/02.jpg|yandex_disk://kpp_photos/56_avtomaticheskaya_kpp_lexus_rx400_mhu38/photos/04.jpg</t>
         </is>
       </c>
       <c r="X60" t="inlineStr">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/57_avtomaticheskaya_kpp_mazda_cx_7_er19/photos/01.jpg|yandex_disk://коробки передач на авито/57_avtomaticheskaya_kpp_mazda_cx_7_er19/photos/02.jpg|yandex_disk://коробки передач на авито/57_avtomaticheskaya_kpp_mazda_cx_7_er19/photos/03.jpg|yandex_disk://коробки передач на авито/57_avtomaticheskaya_kpp_mazda_cx_7_er19/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/57_avtomaticheskaya_kpp_mazda_cx_7_er19/photos/01.jpg|yandex_disk://kpp_photos/57_avtomaticheskaya_kpp_mazda_cx_7_er19/photos/02.jpg|yandex_disk://kpp_photos/57_avtomaticheskaya_kpp_mazda_cx_7_er19/photos/03.jpg|yandex_disk://kpp_photos/57_avtomaticheskaya_kpp_mazda_cx_7_er19/photos/04.jpg</t>
         </is>
       </c>
       <c r="X61" t="inlineStr">
@@ -6836,7 +6836,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/58_avtomaticheskaya_kpp_mazda_atenza_ghefw/photos/01.jpg|yandex_disk://коробки передач на авито/58_avtomaticheskaya_kpp_mazda_atenza_ghefw/photos/02.jpg|yandex_disk://коробки передач на авито/58_avtomaticheskaya_kpp_mazda_atenza_ghefw/photos/03.jpg|yandex_disk://коробки передач на авито/58_avtomaticheskaya_kpp_mazda_atenza_ghefw/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/58_avtomaticheskaya_kpp_mazda_atenza_ghefw/photos/01.jpg|yandex_disk://kpp_photos/58_avtomaticheskaya_kpp_mazda_atenza_ghefw/photos/02.jpg|yandex_disk://kpp_photos/58_avtomaticheskaya_kpp_mazda_atenza_ghefw/photos/03.jpg|yandex_disk://kpp_photos/58_avtomaticheskaya_kpp_mazda_atenza_ghefw/photos/04.jpg</t>
         </is>
       </c>
       <c r="X62" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/59_avtomaticheskaya_kpp_mazda_mazda3_bm/photos/01.jpg|yandex_disk://коробки передач на авито/59_avtomaticheskaya_kpp_mazda_mazda3_bm/photos/02.jpg|yandex_disk://коробки передач на авито/59_avtomaticheskaya_kpp_mazda_mazda3_bm/photos/03.jpg|yandex_disk://коробки передач на авито/59_avtomaticheskaya_kpp_mazda_mazda3_bm/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/59_avtomaticheskaya_kpp_mazda_mazda3_bm/photos/01.jpg|yandex_disk://kpp_photos/59_avtomaticheskaya_kpp_mazda_mazda3_bm/photos/02.jpg|yandex_disk://kpp_photos/59_avtomaticheskaya_kpp_mazda_mazda3_bm/photos/03.jpg|yandex_disk://kpp_photos/59_avtomaticheskaya_kpp_mazda_mazda3_bm/photos/04.jpg</t>
         </is>
       </c>
       <c r="X63" t="inlineStr">
@@ -7016,7 +7016,7 @@
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/60_avtomaticheskaya_kpp_mazda_atenza_gg3s/photos/01.jpg|yandex_disk://коробки передач на авито/60_avtomaticheskaya_kpp_mazda_atenza_gg3s/photos/02.jpg|yandex_disk://коробки передач на авито/60_avtomaticheskaya_kpp_mazda_atenza_gg3s/photos/03.jpg|yandex_disk://коробки передач на авито/60_avtomaticheskaya_kpp_mazda_atenza_gg3s/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/60_avtomaticheskaya_kpp_mazda_atenza_gg3s/photos/01.jpg|yandex_disk://kpp_photos/60_avtomaticheskaya_kpp_mazda_atenza_gg3s/photos/02.jpg|yandex_disk://kpp_photos/60_avtomaticheskaya_kpp_mazda_atenza_gg3s/photos/03.jpg|yandex_disk://kpp_photos/60_avtomaticheskaya_kpp_mazda_atenza_gg3s/photos/04.jpg</t>
         </is>
       </c>
       <c r="X64" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/61_avtomaticheskaya_kpp_mazda_mpv_ly3p/photos/01.jpg|yandex_disk://коробки передач на авито/61_avtomaticheskaya_kpp_mazda_mpv_ly3p/photos/02.jpg|yandex_disk://коробки передач на авито/61_avtomaticheskaya_kpp_mazda_mpv_ly3p/photos/03.jpg|yandex_disk://коробки передач на авито/61_avtomaticheskaya_kpp_mazda_mpv_ly3p/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/61_avtomaticheskaya_kpp_mazda_mpv_ly3p/photos/01.jpg|yandex_disk://kpp_photos/61_avtomaticheskaya_kpp_mazda_mpv_ly3p/photos/02.jpg|yandex_disk://kpp_photos/61_avtomaticheskaya_kpp_mazda_mpv_ly3p/photos/03.jpg|yandex_disk://kpp_photos/61_avtomaticheskaya_kpp_mazda_mpv_ly3p/photos/04.jpg</t>
         </is>
       </c>
       <c r="X65" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/62_avtomaticheskaya_kpp_mazda_axela_bkep/photos/01.jpg|yandex_disk://коробки передач на авито/62_avtomaticheskaya_kpp_mazda_axela_bkep/photos/02.jpg|yandex_disk://коробки передач на авито/62_avtomaticheskaya_kpp_mazda_axela_bkep/photos/03.jpg|yandex_disk://коробки передач на авито/62_avtomaticheskaya_kpp_mazda_axela_bkep/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/62_avtomaticheskaya_kpp_mazda_axela_bkep/photos/01.jpg|yandex_disk://kpp_photos/62_avtomaticheskaya_kpp_mazda_axela_bkep/photos/02.jpg|yandex_disk://kpp_photos/62_avtomaticheskaya_kpp_mazda_axela_bkep/photos/03.jpg|yandex_disk://kpp_photos/62_avtomaticheskaya_kpp_mazda_axela_bkep/photos/04.jpg</t>
         </is>
       </c>
       <c r="X66" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/63_avtomaticheskaya_kpp_mazda_axela_bl5fw/photos/01.jpg|yandex_disk://коробки передач на авито/63_avtomaticheskaya_kpp_mazda_axela_bl5fw/photos/02.jpg|yandex_disk://коробки передач на авито/63_avtomaticheskaya_kpp_mazda_axela_bl5fw/photos/03.jpg|yandex_disk://коробки передач на авито/63_avtomaticheskaya_kpp_mazda_axela_bl5fw/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/63_avtomaticheskaya_kpp_mazda_axela_bl5fw/photos/01.jpg|yandex_disk://kpp_photos/63_avtomaticheskaya_kpp_mazda_axela_bl5fw/photos/02.jpg|yandex_disk://kpp_photos/63_avtomaticheskaya_kpp_mazda_axela_bl5fw/photos/03.jpg|yandex_disk://kpp_photos/63_avtomaticheskaya_kpp_mazda_axela_bl5fw/photos/04.jpg</t>
         </is>
       </c>
       <c r="X67" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/64_avtomaticheskaya_kpp_mazda_demio_de3fs/photos/01.jpg|yandex_disk://коробки передач на авито/64_avtomaticheskaya_kpp_mazda_demio_de3fs/photos/03.jpg|yandex_disk://коробки передач на авито/64_avtomaticheskaya_kpp_mazda_demio_de3fs/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/64_avtomaticheskaya_kpp_mazda_demio_de3fs/photos/01.jpg|yandex_disk://kpp_photos/64_avtomaticheskaya_kpp_mazda_demio_de3fs/photos/03.jpg|yandex_disk://kpp_photos/64_avtomaticheskaya_kpp_mazda_demio_de3fs/photos/04.jpg</t>
         </is>
       </c>
       <c r="X68" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/65_mehanicheskaya_kpp_mazda_demio_dy3w/photos/01.jpg|yandex_disk://коробки передач на авито/65_mehanicheskaya_kpp_mazda_demio_dy3w/photos/02.jpg|yandex_disk://коробки передач на авито/65_mehanicheskaya_kpp_mazda_demio_dy3w/photos/03.jpg|yandex_disk://коробки передач на авито/65_mehanicheskaya_kpp_mazda_demio_dy3w/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/65_mehanicheskaya_kpp_mazda_demio_dy3w/photos/01.jpg|yandex_disk://kpp_photos/65_mehanicheskaya_kpp_mazda_demio_dy3w/photos/02.jpg|yandex_disk://kpp_photos/65_mehanicheskaya_kpp_mazda_demio_dy3w/photos/03.jpg|yandex_disk://kpp_photos/65_mehanicheskaya_kpp_mazda_demio_dy3w/photos/04.jpg</t>
         </is>
       </c>
       <c r="X69" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/66_avtomaticheskaya_kpp_mercedes_benz_gl_class_x164/photos/01.jpg|yandex_disk://коробки передач на авито/66_avtomaticheskaya_kpp_mercedes_benz_gl_class_x164/photos/02.jpg|yandex_disk://коробки передач на авито/66_avtomaticheskaya_kpp_mercedes_benz_gl_class_x164/photos/03.jpg|yandex_disk://коробки передач на авито/66_avtomaticheskaya_kpp_mercedes_benz_gl_class_x164/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/66_avtomaticheskaya_kpp_mercedes_benz_gl_class_x164/photos/01.jpg|yandex_disk://kpp_photos/66_avtomaticheskaya_kpp_mercedes_benz_gl_class_x164/photos/02.jpg|yandex_disk://kpp_photos/66_avtomaticheskaya_kpp_mercedes_benz_gl_class_x164/photos/03.jpg|yandex_disk://kpp_photos/66_avtomaticheskaya_kpp_mercedes_benz_gl_class_x164/photos/04.jpg</t>
         </is>
       </c>
       <c r="X70" t="inlineStr">
@@ -7643,7 +7643,7 @@
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/67_avtomaticheskaya_kpp_mercedes_benz_c_class_w204/photos/01.jpg|yandex_disk://коробки передач на авито/67_avtomaticheskaya_kpp_mercedes_benz_c_class_w204/photos/02.jpg|yandex_disk://коробки передач на авито/67_avtomaticheskaya_kpp_mercedes_benz_c_class_w204/photos/03.jpg|yandex_disk://коробки передач на авито/67_avtomaticheskaya_kpp_mercedes_benz_c_class_w204/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/67_avtomaticheskaya_kpp_mercedes_benz_c_class_w204/photos/01.jpg|yandex_disk://kpp_photos/67_avtomaticheskaya_kpp_mercedes_benz_c_class_w204/photos/02.jpg|yandex_disk://kpp_photos/67_avtomaticheskaya_kpp_mercedes_benz_c_class_w204/photos/03.jpg|yandex_disk://kpp_photos/67_avtomaticheskaya_kpp_mercedes_benz_c_class_w204/photos/04.jpg</t>
         </is>
       </c>
       <c r="X71" t="inlineStr">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/68_avtomaticheskaya_kpp_mercedes_benz_e_class_w210/photos/01.jpg|yandex_disk://коробки передач на авито/68_avtomaticheskaya_kpp_mercedes_benz_e_class_w210/photos/02.jpg|yandex_disk://коробки передач на авито/68_avtomaticheskaya_kpp_mercedes_benz_e_class_w210/photos/03.jpg|yandex_disk://коробки передач на авито/68_avtomaticheskaya_kpp_mercedes_benz_e_class_w210/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/68_avtomaticheskaya_kpp_mercedes_benz_e_class_w210/photos/01.jpg|yandex_disk://kpp_photos/68_avtomaticheskaya_kpp_mercedes_benz_e_class_w210/photos/02.jpg|yandex_disk://kpp_photos/68_avtomaticheskaya_kpp_mercedes_benz_e_class_w210/photos/03.jpg|yandex_disk://kpp_photos/68_avtomaticheskaya_kpp_mercedes_benz_e_class_w210/photos/04.jpg</t>
         </is>
       </c>
       <c r="X72" t="inlineStr">
@@ -7822,7 +7822,7 @@
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/69_avtomaticheskaya_kpp_mitsubishi_lancer_cs7a/photos/01.jpg|yandex_disk://коробки передач на авито/69_avtomaticheskaya_kpp_mitsubishi_lancer_cs7a/photos/02.jpg|yandex_disk://коробки передач на авито/69_avtomaticheskaya_kpp_mitsubishi_lancer_cs7a/photos/03.jpg|yandex_disk://коробки передач на авито/69_avtomaticheskaya_kpp_mitsubishi_lancer_cs7a/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/69_avtomaticheskaya_kpp_mitsubishi_lancer_cs7a/photos/01.jpg|yandex_disk://kpp_photos/69_avtomaticheskaya_kpp_mitsubishi_lancer_cs7a/photos/02.jpg|yandex_disk://kpp_photos/69_avtomaticheskaya_kpp_mitsubishi_lancer_cs7a/photos/03.jpg|yandex_disk://kpp_photos/69_avtomaticheskaya_kpp_mitsubishi_lancer_cs7a/photos/04.jpg</t>
         </is>
       </c>
       <c r="X73" t="inlineStr">
@@ -7912,7 +7912,7 @@
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/70_mehanicheskaya_kpp_mitsubishi_lancer_cy4a/photos/01.jpg|yandex_disk://коробки передач на авито/70_mehanicheskaya_kpp_mitsubishi_lancer_cy4a/photos/02.jpg|yandex_disk://коробки передач на авито/70_mehanicheskaya_kpp_mitsubishi_lancer_cy4a/photos/03.jpg|yandex_disk://коробки передач на авито/70_mehanicheskaya_kpp_mitsubishi_lancer_cy4a/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/70_mehanicheskaya_kpp_mitsubishi_lancer_cy4a/photos/01.jpg|yandex_disk://kpp_photos/70_mehanicheskaya_kpp_mitsubishi_lancer_cy4a/photos/02.jpg|yandex_disk://kpp_photos/70_mehanicheskaya_kpp_mitsubishi_lancer_cy4a/photos/03.jpg|yandex_disk://kpp_photos/70_mehanicheskaya_kpp_mitsubishi_lancer_cy4a/photos/04.jpg</t>
         </is>
       </c>
       <c r="X74" t="inlineStr">
@@ -8002,7 +8002,7 @@
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/71_mehanicheskaya_kpp_mitsubishi_canter_fb51ab/photos/01.jpg|yandex_disk://коробки передач на авито/71_mehanicheskaya_kpp_mitsubishi_canter_fb51ab/photos/02.jpg|yandex_disk://коробки передач на авито/71_mehanicheskaya_kpp_mitsubishi_canter_fb51ab/photos/03.jpg|yandex_disk://коробки передач на авито/71_mehanicheskaya_kpp_mitsubishi_canter_fb51ab/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/71_mehanicheskaya_kpp_mitsubishi_canter_fb51ab/photos/01.jpg|yandex_disk://kpp_photos/71_mehanicheskaya_kpp_mitsubishi_canter_fb51ab/photos/02.jpg|yandex_disk://kpp_photos/71_mehanicheskaya_kpp_mitsubishi_canter_fb51ab/photos/03.jpg|yandex_disk://kpp_photos/71_mehanicheskaya_kpp_mitsubishi_canter_fb51ab/photos/04.jpg</t>
         </is>
       </c>
       <c r="X75" t="inlineStr">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/72_avtomaticheskaya_kpp_nissan_x_trail_nt32/photos/01.jpg|yandex_disk://коробки передач на авито/72_avtomaticheskaya_kpp_nissan_x_trail_nt32/photos/02.jpg|yandex_disk://коробки передач на авито/72_avtomaticheskaya_kpp_nissan_x_trail_nt32/photos/03.jpg|yandex_disk://коробки передач на авито/72_avtomaticheskaya_kpp_nissan_x_trail_nt32/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/72_avtomaticheskaya_kpp_nissan_x_trail_nt32/photos/01.jpg|yandex_disk://kpp_photos/72_avtomaticheskaya_kpp_nissan_x_trail_nt32/photos/02.jpg|yandex_disk://kpp_photos/72_avtomaticheskaya_kpp_nissan_x_trail_nt32/photos/03.jpg|yandex_disk://kpp_photos/72_avtomaticheskaya_kpp_nissan_x_trail_nt32/photos/04.jpg</t>
         </is>
       </c>
       <c r="X76" t="inlineStr">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/73_avtomaticheskaya_kpp_nissan_juke_yf15/photos/01.jpg|yandex_disk://коробки передач на авито/73_avtomaticheskaya_kpp_nissan_juke_yf15/photos/02.jpg|yandex_disk://коробки передач на авито/73_avtomaticheskaya_kpp_nissan_juke_yf15/photos/03.jpg|yandex_disk://коробки передач на авито/73_avtomaticheskaya_kpp_nissan_juke_yf15/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/73_avtomaticheskaya_kpp_nissan_juke_yf15/photos/01.jpg|yandex_disk://kpp_photos/73_avtomaticheskaya_kpp_nissan_juke_yf15/photos/02.jpg|yandex_disk://kpp_photos/73_avtomaticheskaya_kpp_nissan_juke_yf15/photos/03.jpg|yandex_disk://kpp_photos/73_avtomaticheskaya_kpp_nissan_juke_yf15/photos/04.jpg</t>
         </is>
       </c>
       <c r="X77" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/74_avtomaticheskaya_kpp_nissan_qashqai_j10/photos/01.jpg|yandex_disk://коробки передач на авито/74_avtomaticheskaya_kpp_nissan_qashqai_j10/photos/02.jpg|yandex_disk://коробки передач на авито/74_avtomaticheskaya_kpp_nissan_qashqai_j10/photos/03.jpg|yandex_disk://коробки передач на авито/74_avtomaticheskaya_kpp_nissan_qashqai_j10/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/74_avtomaticheskaya_kpp_nissan_qashqai_j10/photos/01.jpg|yandex_disk://kpp_photos/74_avtomaticheskaya_kpp_nissan_qashqai_j10/photos/02.jpg|yandex_disk://kpp_photos/74_avtomaticheskaya_kpp_nissan_qashqai_j10/photos/03.jpg|yandex_disk://kpp_photos/74_avtomaticheskaya_kpp_nissan_qashqai_j10/photos/04.jpg</t>
         </is>
       </c>
       <c r="X78" t="inlineStr">
@@ -8362,7 +8362,7 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/75_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/01.jpg|yandex_disk://коробки передач на авито/75_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/02.jpg|yandex_disk://коробки передач на авито/75_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/03.jpg|yandex_disk://коробки передач на авито/75_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/75_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/01.jpg|yandex_disk://kpp_photos/75_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/02.jpg|yandex_disk://kpp_photos/75_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/03.jpg|yandex_disk://kpp_photos/75_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/04.jpg</t>
         </is>
       </c>
       <c r="X79" t="inlineStr">
@@ -8452,7 +8452,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/76_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/01.jpg|yandex_disk://коробки передач на авито/76_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/02.jpg|yandex_disk://коробки передач на авито/76_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/03.jpg|yandex_disk://коробки передач на авито/76_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/76_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/01.jpg|yandex_disk://kpp_photos/76_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/02.jpg|yandex_disk://kpp_photos/76_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/03.jpg|yandex_disk://kpp_photos/76_avtomaticheskaya_kpp_nissan_qashqai_2_j10/photos/04.jpg</t>
         </is>
       </c>
       <c r="X80" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/77_avtomaticheskaya_kpp_nissan_ad_vzny12/photos/01.jpg|yandex_disk://коробки передач на авито/77_avtomaticheskaya_kpp_nissan_ad_vzny12/photos/02.jpg|yandex_disk://коробки передач на авито/77_avtomaticheskaya_kpp_nissan_ad_vzny12/photos/03.jpg|yandex_disk://коробки передач на авито/77_avtomaticheskaya_kpp_nissan_ad_vzny12/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/77_avtomaticheskaya_kpp_nissan_ad_vzny12/photos/01.jpg|yandex_disk://kpp_photos/77_avtomaticheskaya_kpp_nissan_ad_vzny12/photos/02.jpg|yandex_disk://kpp_photos/77_avtomaticheskaya_kpp_nissan_ad_vzny12/photos/03.jpg|yandex_disk://kpp_photos/77_avtomaticheskaya_kpp_nissan_ad_vzny12/photos/04.jpg</t>
         </is>
       </c>
       <c r="X81" t="inlineStr">
@@ -8632,7 +8632,7 @@
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/78_avtomaticheskaya_kpp_nissan_serena_cc25/photos/01.jpg|yandex_disk://коробки передач на авито/78_avtomaticheskaya_kpp_nissan_serena_cc25/photos/03.jpg|yandex_disk://коробки передач на авито/78_avtomaticheskaya_kpp_nissan_serena_cc25/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/78_avtomaticheskaya_kpp_nissan_serena_cc25/photos/01.jpg|yandex_disk://kpp_photos/78_avtomaticheskaya_kpp_nissan_serena_cc25/photos/03.jpg|yandex_disk://kpp_photos/78_avtomaticheskaya_kpp_nissan_serena_cc25/photos/04.jpg</t>
         </is>
       </c>
       <c r="X82" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/79_avtomaticheskaya_kpp_peugeot_4008_bu/photos/01.jpg|yandex_disk://коробки передач на авито/79_avtomaticheskaya_kpp_peugeot_4008_bu/photos/02.jpg|yandex_disk://коробки передач на авито/79_avtomaticheskaya_kpp_peugeot_4008_bu/photos/03.jpg|yandex_disk://коробки передач на авито/79_avtomaticheskaya_kpp_peugeot_4008_bu/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/79_avtomaticheskaya_kpp_peugeot_4008_bu/photos/01.jpg|yandex_disk://kpp_photos/79_avtomaticheskaya_kpp_peugeot_4008_bu/photos/02.jpg|yandex_disk://kpp_photos/79_avtomaticheskaya_kpp_peugeot_4008_bu/photos/03.jpg|yandex_disk://kpp_photos/79_avtomaticheskaya_kpp_peugeot_4008_bu/photos/04.jpg</t>
         </is>
       </c>
       <c r="X83" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/80_avtomaticheskaya_kpp_peugeot_4008_bu/photos/01.jpg|yandex_disk://коробки передач на авито/80_avtomaticheskaya_kpp_peugeot_4008_bu/photos/02.jpg|yandex_disk://коробки передач на авито/80_avtomaticheskaya_kpp_peugeot_4008_bu/photos/03.jpg|yandex_disk://коробки передач на авито/80_avtomaticheskaya_kpp_peugeot_4008_bu/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/80_avtomaticheskaya_kpp_peugeot_4008_bu/photos/01.jpg|yandex_disk://kpp_photos/80_avtomaticheskaya_kpp_peugeot_4008_bu/photos/02.jpg|yandex_disk://kpp_photos/80_avtomaticheskaya_kpp_peugeot_4008_bu/photos/03.jpg|yandex_disk://kpp_photos/80_avtomaticheskaya_kpp_peugeot_4008_bu/photos/04.jpg</t>
         </is>
       </c>
       <c r="X84" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/81_avtomaticheskaya_kpp_peugeot_4008_bu/photos/01.jpg|yandex_disk://коробки передач на авито/81_avtomaticheskaya_kpp_peugeot_4008_bu/photos/02.jpg|yandex_disk://коробки передач на авито/81_avtomaticheskaya_kpp_peugeot_4008_bu/photos/03.jpg|yandex_disk://коробки передач на авито/81_avtomaticheskaya_kpp_peugeot_4008_bu/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/81_avtomaticheskaya_kpp_peugeot_4008_bu/photos/01.jpg|yandex_disk://kpp_photos/81_avtomaticheskaya_kpp_peugeot_4008_bu/photos/02.jpg|yandex_disk://kpp_photos/81_avtomaticheskaya_kpp_peugeot_4008_bu/photos/03.jpg|yandex_disk://kpp_photos/81_avtomaticheskaya_kpp_peugeot_4008_bu/photos/04.jpg</t>
         </is>
       </c>
       <c r="X85" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/82_mehanicheskaya_kpp_peugeot_partner_tepee_b9/photos/01.jpg|yandex_disk://коробки передач на авито/82_mehanicheskaya_kpp_peugeot_partner_tepee_b9/photos/02.jpg|yandex_disk://коробки передач на авито/82_mehanicheskaya_kpp_peugeot_partner_tepee_b9/photos/03.jpg|yandex_disk://коробки передач на авито/82_mehanicheskaya_kpp_peugeot_partner_tepee_b9/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/82_mehanicheskaya_kpp_peugeot_partner_tepee_b9/photos/01.jpg|yandex_disk://kpp_photos/82_mehanicheskaya_kpp_peugeot_partner_tepee_b9/photos/02.jpg|yandex_disk://kpp_photos/82_mehanicheskaya_kpp_peugeot_partner_tepee_b9/photos/03.jpg|yandex_disk://kpp_photos/82_mehanicheskaya_kpp_peugeot_partner_tepee_b9/photos/04.jpg</t>
         </is>
       </c>
       <c r="X86" t="inlineStr">
@@ -9081,7 +9081,7 @@
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/83_avtomaticheskaya_kpp_renault_trafic_jl/photos/01.jpg|yandex_disk://коробки передач на авито/83_avtomaticheskaya_kpp_renault_trafic_jl/photos/02.jpg|yandex_disk://коробки передач на авито/83_avtomaticheskaya_kpp_renault_trafic_jl/photos/03.jpg|yandex_disk://коробки передач на авито/83_avtomaticheskaya_kpp_renault_trafic_jl/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/83_avtomaticheskaya_kpp_renault_trafic_jl/photos/01.jpg|yandex_disk://kpp_photos/83_avtomaticheskaya_kpp_renault_trafic_jl/photos/02.jpg|yandex_disk://kpp_photos/83_avtomaticheskaya_kpp_renault_trafic_jl/photos/03.jpg|yandex_disk://kpp_photos/83_avtomaticheskaya_kpp_renault_trafic_jl/photos/04.jpg</t>
         </is>
       </c>
       <c r="X87" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/84_avtomaticheskaya_kpp_renault_kangoo_kw0/photos/01.jpg|yandex_disk://коробки передач на авито/84_avtomaticheskaya_kpp_renault_kangoo_kw0/photos/02.jpg|yandex_disk://коробки передач на авито/84_avtomaticheskaya_kpp_renault_kangoo_kw0/photos/03.jpg|yandex_disk://коробки передач на авито/84_avtomaticheskaya_kpp_renault_kangoo_kw0/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/84_avtomaticheskaya_kpp_renault_kangoo_kw0/photos/01.jpg|yandex_disk://kpp_photos/84_avtomaticheskaya_kpp_renault_kangoo_kw0/photos/02.jpg|yandex_disk://kpp_photos/84_avtomaticheskaya_kpp_renault_kangoo_kw0/photos/03.jpg|yandex_disk://kpp_photos/84_avtomaticheskaya_kpp_renault_kangoo_kw0/photos/04.jpg</t>
         </is>
       </c>
       <c r="X88" t="inlineStr">
@@ -9261,7 +9261,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/85_mehanicheskaya_kpp_renault_kangoo_kc/photos/01.jpg|yandex_disk://коробки передач на авито/85_mehanicheskaya_kpp_renault_kangoo_kc/photos/02.jpg|yandex_disk://коробки передач на авито/85_mehanicheskaya_kpp_renault_kangoo_kc/photos/03.jpg|yandex_disk://коробки передач на авито/85_mehanicheskaya_kpp_renault_kangoo_kc/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/85_mehanicheskaya_kpp_renault_kangoo_kc/photos/01.jpg|yandex_disk://kpp_photos/85_mehanicheskaya_kpp_renault_kangoo_kc/photos/02.jpg|yandex_disk://kpp_photos/85_mehanicheskaya_kpp_renault_kangoo_kc/photos/03.jpg|yandex_disk://kpp_photos/85_mehanicheskaya_kpp_renault_kangoo_kc/photos/04.jpg</t>
         </is>
       </c>
       <c r="X89" t="inlineStr">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/86_mehanicheskaya_kpp_renault_megane_bm/photos/01.jpg|yandex_disk://коробки передач на авито/86_mehanicheskaya_kpp_renault_megane_bm/photos/02.jpg|yandex_disk://коробки передач на авито/86_mehanicheskaya_kpp_renault_megane_bm/photos/03.jpg|yandex_disk://коробки передач на авито/86_mehanicheskaya_kpp_renault_megane_bm/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/86_mehanicheskaya_kpp_renault_megane_bm/photos/01.jpg|yandex_disk://kpp_photos/86_mehanicheskaya_kpp_renault_megane_bm/photos/02.jpg|yandex_disk://kpp_photos/86_mehanicheskaya_kpp_renault_megane_bm/photos/03.jpg|yandex_disk://kpp_photos/86_mehanicheskaya_kpp_renault_megane_bm/photos/04.jpg</t>
         </is>
       </c>
       <c r="X90" t="inlineStr">
@@ -9440,7 +9440,7 @@
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/87_mehanicheskaya_kpp_renault_kangoo_kw0/photos/01.jpg|yandex_disk://коробки передач на авито/87_mehanicheskaya_kpp_renault_kangoo_kw0/photos/02.jpg|yandex_disk://коробки передач на авито/87_mehanicheskaya_kpp_renault_kangoo_kw0/photos/03.jpg|yandex_disk://коробки передач на авито/87_mehanicheskaya_kpp_renault_kangoo_kw0/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/87_mehanicheskaya_kpp_renault_kangoo_kw0/photos/01.jpg|yandex_disk://kpp_photos/87_mehanicheskaya_kpp_renault_kangoo_kw0/photos/02.jpg|yandex_disk://kpp_photos/87_mehanicheskaya_kpp_renault_kangoo_kw0/photos/03.jpg|yandex_disk://kpp_photos/87_mehanicheskaya_kpp_renault_kangoo_kw0/photos/04.jpg</t>
         </is>
       </c>
       <c r="X91" t="inlineStr">
@@ -9530,7 +9530,7 @@
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/88_mehanicheskaya_kpp_skoda_octavia_a5_1z3/photos/01.jpg|yandex_disk://коробки передач на авито/88_mehanicheskaya_kpp_skoda_octavia_a5_1z3/photos/02.jpg|yandex_disk://коробки передач на авито/88_mehanicheskaya_kpp_skoda_octavia_a5_1z3/photos/03.jpg|yandex_disk://коробки передач на авито/88_mehanicheskaya_kpp_skoda_octavia_a5_1z3/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/88_mehanicheskaya_kpp_skoda_octavia_a5_1z3/photos/01.jpg|yandex_disk://kpp_photos/88_mehanicheskaya_kpp_skoda_octavia_a5_1z3/photos/02.jpg|yandex_disk://kpp_photos/88_mehanicheskaya_kpp_skoda_octavia_a5_1z3/photos/03.jpg|yandex_disk://kpp_photos/88_mehanicheskaya_kpp_skoda_octavia_a5_1z3/photos/04.jpg</t>
         </is>
       </c>
       <c r="X92" t="inlineStr">
@@ -9620,7 +9620,7 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/89_avtomaticheskaya_kpp_ssangyong_actyon_ck/photos/01.jpg|yandex_disk://коробки передач на авито/89_avtomaticheskaya_kpp_ssangyong_actyon_ck/photos/02.jpg|yandex_disk://коробки передач на авито/89_avtomaticheskaya_kpp_ssangyong_actyon_ck/photos/03.jpg|yandex_disk://коробки передач на авито/89_avtomaticheskaya_kpp_ssangyong_actyon_ck/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/89_avtomaticheskaya_kpp_ssangyong_actyon_ck/photos/01.jpg|yandex_disk://kpp_photos/89_avtomaticheskaya_kpp_ssangyong_actyon_ck/photos/02.jpg|yandex_disk://kpp_photos/89_avtomaticheskaya_kpp_ssangyong_actyon_ck/photos/03.jpg|yandex_disk://kpp_photos/89_avtomaticheskaya_kpp_ssangyong_actyon_ck/photos/04.jpg</t>
         </is>
       </c>
       <c r="X93" t="inlineStr">
@@ -9709,7 +9709,7 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/90_avtomaticheskaya_kpp_subaru_tribeca_wxf/photos/01.jpg|yandex_disk://коробки передач на авито/90_avtomaticheskaya_kpp_subaru_tribeca_wxf/photos/02.jpg|yandex_disk://коробки передач на авито/90_avtomaticheskaya_kpp_subaru_tribeca_wxf/photos/03.jpg|yandex_disk://коробки передач на авито/90_avtomaticheskaya_kpp_subaru_tribeca_wxf/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/90_avtomaticheskaya_kpp_subaru_tribeca_wxf/photos/01.jpg|yandex_disk://kpp_photos/90_avtomaticheskaya_kpp_subaru_tribeca_wxf/photos/02.jpg|yandex_disk://kpp_photos/90_avtomaticheskaya_kpp_subaru_tribeca_wxf/photos/03.jpg|yandex_disk://kpp_photos/90_avtomaticheskaya_kpp_subaru_tribeca_wxf/photos/04.jpg</t>
         </is>
       </c>
       <c r="X94" t="inlineStr">
@@ -9799,7 +9799,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/91_avtomaticheskaya_kpp_subaru_impreza_gp7/photos/01.jpg|yandex_disk://коробки передач на авито/91_avtomaticheskaya_kpp_subaru_impreza_gp7/photos/03.jpg|yandex_disk://коробки передач на авито/91_avtomaticheskaya_kpp_subaru_impreza_gp7/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/91_avtomaticheskaya_kpp_subaru_impreza_gp7/photos/01.jpg|yandex_disk://kpp_photos/91_avtomaticheskaya_kpp_subaru_impreza_gp7/photos/03.jpg|yandex_disk://kpp_photos/91_avtomaticheskaya_kpp_subaru_impreza_gp7/photos/04.jpg</t>
         </is>
       </c>
       <c r="X95" t="inlineStr">
@@ -9889,7 +9889,7 @@
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/92_avtomaticheskaya_kpp_subaru_legacy_bm9/photos/01.jpg|yandex_disk://коробки передач на авито/92_avtomaticheskaya_kpp_subaru_legacy_bm9/photos/03.jpg|yandex_disk://коробки передач на авито/92_avtomaticheskaya_kpp_subaru_legacy_bm9/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/92_avtomaticheskaya_kpp_subaru_legacy_bm9/photos/01.jpg|yandex_disk://kpp_photos/92_avtomaticheskaya_kpp_subaru_legacy_bm9/photos/03.jpg|yandex_disk://kpp_photos/92_avtomaticheskaya_kpp_subaru_legacy_bm9/photos/04.jpg</t>
         </is>
       </c>
       <c r="X96" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/93_avtomaticheskaya_kpp_subaru_impreza_gp2/photos/01.jpg|yandex_disk://коробки передач на авито/93_avtomaticheskaya_kpp_subaru_impreza_gp2/photos/02.jpg|yandex_disk://коробки передач на авито/93_avtomaticheskaya_kpp_subaru_impreza_gp2/photos/03.jpg|yandex_disk://коробки передач на авито/93_avtomaticheskaya_kpp_subaru_impreza_gp2/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/93_avtomaticheskaya_kpp_subaru_impreza_gp2/photos/01.jpg|yandex_disk://kpp_photos/93_avtomaticheskaya_kpp_subaru_impreza_gp2/photos/02.jpg|yandex_disk://kpp_photos/93_avtomaticheskaya_kpp_subaru_impreza_gp2/photos/03.jpg|yandex_disk://kpp_photos/93_avtomaticheskaya_kpp_subaru_impreza_gp2/photos/04.jpg</t>
         </is>
       </c>
       <c r="X97" t="inlineStr">
@@ -10067,7 +10067,7 @@
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/94_mehanicheskaya_kpp_subaru_impreza_gg3/photos/01.jpg|yandex_disk://коробки передач на авито/94_mehanicheskaya_kpp_subaru_impreza_gg3/photos/02.jpg|yandex_disk://коробки передач на авито/94_mehanicheskaya_kpp_subaru_impreza_gg3/photos/03.jpg|yandex_disk://коробки передач на авито/94_mehanicheskaya_kpp_subaru_impreza_gg3/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/94_mehanicheskaya_kpp_subaru_impreza_gg3/photos/01.jpg|yandex_disk://kpp_photos/94_mehanicheskaya_kpp_subaru_impreza_gg3/photos/02.jpg|yandex_disk://kpp_photos/94_mehanicheskaya_kpp_subaru_impreza_gg3/photos/03.jpg|yandex_disk://kpp_photos/94_mehanicheskaya_kpp_subaru_impreza_gg3/photos/04.jpg</t>
         </is>
       </c>
       <c r="X98" t="inlineStr">
@@ -10157,7 +10157,7 @@
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/95_avtomaticheskaya_kpp_suzuki_sx4_jyaa2/photos/01.jpg|yandex_disk://коробки передач на авито/95_avtomaticheskaya_kpp_suzuki_sx4_jyaa2/photos/03.jpg|yandex_disk://коробки передач на авито/95_avtomaticheskaya_kpp_suzuki_sx4_jyaa2/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/95_avtomaticheskaya_kpp_suzuki_sx4_jyaa2/photos/01.jpg|yandex_disk://kpp_photos/95_avtomaticheskaya_kpp_suzuki_sx4_jyaa2/photos/03.jpg|yandex_disk://kpp_photos/95_avtomaticheskaya_kpp_suzuki_sx4_jyaa2/photos/04.jpg</t>
         </is>
       </c>
       <c r="X99" t="inlineStr">
@@ -10247,7 +10247,7 @@
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/96_avtomaticheskaya_kpp_suzuki_vitara_ly/photos/01.jpg|yandex_disk://коробки передач на авито/96_avtomaticheskaya_kpp_suzuki_vitara_ly/photos/02.jpg|yandex_disk://коробки передач на авито/96_avtomaticheskaya_kpp_suzuki_vitara_ly/photos/03.jpg|yandex_disk://коробки передач на авито/96_avtomaticheskaya_kpp_suzuki_vitara_ly/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/96_avtomaticheskaya_kpp_suzuki_vitara_ly/photos/01.jpg|yandex_disk://kpp_photos/96_avtomaticheskaya_kpp_suzuki_vitara_ly/photos/02.jpg|yandex_disk://kpp_photos/96_avtomaticheskaya_kpp_suzuki_vitara_ly/photos/03.jpg|yandex_disk://kpp_photos/96_avtomaticheskaya_kpp_suzuki_vitara_ly/photos/04.jpg</t>
         </is>
       </c>
       <c r="X100" t="inlineStr">
@@ -10337,7 +10337,7 @@
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/97_avtomaticheskaya_kpp_suzuki_alto_hc11v/photos/01.jpg|yandex_disk://коробки передач на авито/97_avtomaticheskaya_kpp_suzuki_alto_hc11v/photos/02.jpg|yandex_disk://коробки передач на авито/97_avtomaticheskaya_kpp_suzuki_alto_hc11v/photos/03.jpg|yandex_disk://коробки передач на авито/97_avtomaticheskaya_kpp_suzuki_alto_hc11v/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/97_avtomaticheskaya_kpp_suzuki_alto_hc11v/photos/01.jpg|yandex_disk://kpp_photos/97_avtomaticheskaya_kpp_suzuki_alto_hc11v/photos/02.jpg|yandex_disk://kpp_photos/97_avtomaticheskaya_kpp_suzuki_alto_hc11v/photos/03.jpg|yandex_disk://kpp_photos/97_avtomaticheskaya_kpp_suzuki_alto_hc11v/photos/04.jpg</t>
         </is>
       </c>
       <c r="X101" t="inlineStr">
@@ -10427,7 +10427,7 @@
       </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/98_mehanicheskaya_kpp_suzuki_vitara_ly/photos/01.jpg|yandex_disk://коробки передач на авито/98_mehanicheskaya_kpp_suzuki_vitara_ly/photos/02.jpg|yandex_disk://коробки передач на авито/98_mehanicheskaya_kpp_suzuki_vitara_ly/photos/03.jpg|yandex_disk://коробки передач на авито/98_mehanicheskaya_kpp_suzuki_vitara_ly/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/98_mehanicheskaya_kpp_suzuki_vitara_ly/photos/01.jpg|yandex_disk://kpp_photos/98_mehanicheskaya_kpp_suzuki_vitara_ly/photos/02.jpg|yandex_disk://kpp_photos/98_mehanicheskaya_kpp_suzuki_vitara_ly/photos/03.jpg|yandex_disk://kpp_photos/98_mehanicheskaya_kpp_suzuki_vitara_ly/photos/04.jpg</t>
         </is>
       </c>
       <c r="X102" t="inlineStr">
@@ -10516,7 +10516,7 @@
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/99_avtomaticheskaya_kpp_toyota_camry_acv40/photos/01.jpg|yandex_disk://коробки передач на авито/99_avtomaticheskaya_kpp_toyota_camry_acv40/photos/02.jpg|yandex_disk://коробки передач на авито/99_avtomaticheskaya_kpp_toyota_camry_acv40/photos/03.jpg|yandex_disk://коробки передач на авито/99_avtomaticheskaya_kpp_toyota_camry_acv40/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/99_avtomaticheskaya_kpp_toyota_camry_acv40/photos/01.jpg|yandex_disk://kpp_photos/99_avtomaticheskaya_kpp_toyota_camry_acv40/photos/02.jpg|yandex_disk://kpp_photos/99_avtomaticheskaya_kpp_toyota_camry_acv40/photos/03.jpg|yandex_disk://kpp_photos/99_avtomaticheskaya_kpp_toyota_camry_acv40/photos/04.jpg</t>
         </is>
       </c>
       <c r="X103" t="inlineStr">
@@ -10605,7 +10605,7 @@
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/100_avtomaticheskaya_kpp_toyota_camry_acv40/photos/01.jpg|yandex_disk://коробки передач на авито/100_avtomaticheskaya_kpp_toyota_camry_acv40/photos/02.jpg|yandex_disk://коробки передач на авито/100_avtomaticheskaya_kpp_toyota_camry_acv40/photos/03.jpg|yandex_disk://коробки передач на авито/100_avtomaticheskaya_kpp_toyota_camry_acv40/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/100_avtomaticheskaya_kpp_toyota_camry_acv40/photos/01.jpg|yandex_disk://kpp_photos/100_avtomaticheskaya_kpp_toyota_camry_acv40/photos/02.jpg|yandex_disk://kpp_photos/100_avtomaticheskaya_kpp_toyota_camry_acv40/photos/03.jpg|yandex_disk://kpp_photos/100_avtomaticheskaya_kpp_toyota_camry_acv40/photos/04.jpg</t>
         </is>
       </c>
       <c r="X104" t="inlineStr">
@@ -10695,7 +10695,7 @@
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/101_avtomaticheskaya_kpp_toyota_corolla_zre152/photos/01.jpg|yandex_disk://коробки передач на авито/101_avtomaticheskaya_kpp_toyota_corolla_zre152/photos/02.jpg|yandex_disk://коробки передач на авито/101_avtomaticheskaya_kpp_toyota_corolla_zre152/photos/03.jpg|yandex_disk://коробки передач на авито/101_avtomaticheskaya_kpp_toyota_corolla_zre152/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/101_avtomaticheskaya_kpp_toyota_corolla_zre152/photos/01.jpg|yandex_disk://kpp_photos/101_avtomaticheskaya_kpp_toyota_corolla_zre152/photos/02.jpg|yandex_disk://kpp_photos/101_avtomaticheskaya_kpp_toyota_corolla_zre152/photos/03.jpg|yandex_disk://kpp_photos/101_avtomaticheskaya_kpp_toyota_corolla_zre152/photos/04.jpg</t>
         </is>
       </c>
       <c r="X105" t="inlineStr">
@@ -10784,7 +10784,7 @@
       </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/102_avtomaticheskaya_kpp_toyota_c_hr_ngx10/photos/01.jpg|yandex_disk://коробки передач на авито/102_avtomaticheskaya_kpp_toyota_c_hr_ngx10/photos/02.jpg|yandex_disk://коробки передач на авито/102_avtomaticheskaya_kpp_toyota_c_hr_ngx10/photos/03.jpg|yandex_disk://коробки передач на авито/102_avtomaticheskaya_kpp_toyota_c_hr_ngx10/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/102_avtomaticheskaya_kpp_toyota_c_hr_ngx10/photos/01.jpg|yandex_disk://kpp_photos/102_avtomaticheskaya_kpp_toyota_c_hr_ngx10/photos/02.jpg|yandex_disk://kpp_photos/102_avtomaticheskaya_kpp_toyota_c_hr_ngx10/photos/03.jpg|yandex_disk://kpp_photos/102_avtomaticheskaya_kpp_toyota_c_hr_ngx10/photos/04.jpg</t>
         </is>
       </c>
       <c r="X106" t="inlineStr">
@@ -10873,7 +10873,7 @@
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/103_avtomaticheskaya_kpp_toyota_corolla_zre172/photos/01.jpg|yandex_disk://коробки передач на авито/103_avtomaticheskaya_kpp_toyota_corolla_zre172/photos/02.jpg|yandex_disk://коробки передач на авито/103_avtomaticheskaya_kpp_toyota_corolla_zre172/photos/03.jpg|yandex_disk://коробки передач на авито/103_avtomaticheskaya_kpp_toyota_corolla_zre172/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/103_avtomaticheskaya_kpp_toyota_corolla_zre172/photos/01.jpg|yandex_disk://kpp_photos/103_avtomaticheskaya_kpp_toyota_corolla_zre172/photos/02.jpg|yandex_disk://kpp_photos/103_avtomaticheskaya_kpp_toyota_corolla_zre172/photos/03.jpg|yandex_disk://kpp_photos/103_avtomaticheskaya_kpp_toyota_corolla_zre172/photos/04.jpg</t>
         </is>
       </c>
       <c r="X107" t="inlineStr">
@@ -10962,7 +10962,7 @@
       </c>
       <c r="S108" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/104_avtomaticheskaya_kpp_toyota_avensis_zrt272/photos/01.jpg|yandex_disk://коробки передач на авито/104_avtomaticheskaya_kpp_toyota_avensis_zrt272/photos/02.jpg|yandex_disk://коробки передач на авито/104_avtomaticheskaya_kpp_toyota_avensis_zrt272/photos/03.jpg|yandex_disk://коробки передач на авито/104_avtomaticheskaya_kpp_toyota_avensis_zrt272/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/104_avtomaticheskaya_kpp_toyota_avensis_zrt272/photos/01.jpg|yandex_disk://kpp_photos/104_avtomaticheskaya_kpp_toyota_avensis_zrt272/photos/02.jpg|yandex_disk://kpp_photos/104_avtomaticheskaya_kpp_toyota_avensis_zrt272/photos/03.jpg|yandex_disk://kpp_photos/104_avtomaticheskaya_kpp_toyota_avensis_zrt272/photos/04.jpg</t>
         </is>
       </c>
       <c r="X108" t="inlineStr">
@@ -11052,7 +11052,7 @@
       </c>
       <c r="S109" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/105_avtomaticheskaya_kpp_toyota_passo_kgc30/photos/01.jpg|yandex_disk://коробки передач на авито/105_avtomaticheskaya_kpp_toyota_passo_kgc30/photos/02.jpg|yandex_disk://коробки передач на авито/105_avtomaticheskaya_kpp_toyota_passo_kgc30/photos/03.jpg|yandex_disk://коробки передач на авито/105_avtomaticheskaya_kpp_toyota_passo_kgc30/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/105_avtomaticheskaya_kpp_toyota_passo_kgc30/photos/01.jpg|yandex_disk://kpp_photos/105_avtomaticheskaya_kpp_toyota_passo_kgc30/photos/02.jpg|yandex_disk://kpp_photos/105_avtomaticheskaya_kpp_toyota_passo_kgc30/photos/03.jpg|yandex_disk://kpp_photos/105_avtomaticheskaya_kpp_toyota_passo_kgc30/photos/04.jpg</t>
         </is>
       </c>
       <c r="X109" t="inlineStr">
@@ -11141,7 +11141,7 @@
       </c>
       <c r="S110" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/106_mehanicheskaya_kpp_toyota_yaris_ncp10/photos/01.jpg|yandex_disk://коробки передач на авито/106_mehanicheskaya_kpp_toyota_yaris_ncp10/photos/03.jpg|yandex_disk://коробки передач на авито/106_mehanicheskaya_kpp_toyota_yaris_ncp10/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/106_mehanicheskaya_kpp_toyota_yaris_ncp10/photos/01.jpg|yandex_disk://kpp_photos/106_mehanicheskaya_kpp_toyota_yaris_ncp10/photos/03.jpg|yandex_disk://kpp_photos/106_mehanicheskaya_kpp_toyota_yaris_ncp10/photos/04.jpg</t>
         </is>
       </c>
       <c r="X110" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="S111" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/107_avtomaticheskaya_kpp_volkswagen_amarok_2ha/photos/01.jpg|yandex_disk://коробки передач на авито/107_avtomaticheskaya_kpp_volkswagen_amarok_2ha/photos/02.jpg|yandex_disk://коробки передач на авито/107_avtomaticheskaya_kpp_volkswagen_amarok_2ha/photos/03.jpg|yandex_disk://коробки передач на авито/107_avtomaticheskaya_kpp_volkswagen_amarok_2ha/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/107_avtomaticheskaya_kpp_volkswagen_amarok_2ha/photos/01.jpg|yandex_disk://kpp_photos/107_avtomaticheskaya_kpp_volkswagen_amarok_2ha/photos/02.jpg|yandex_disk://kpp_photos/107_avtomaticheskaya_kpp_volkswagen_amarok_2ha/photos/03.jpg|yandex_disk://kpp_photos/107_avtomaticheskaya_kpp_volkswagen_amarok_2ha/photos/04.jpg</t>
         </is>
       </c>
       <c r="X111" t="inlineStr">
@@ -11321,7 +11321,7 @@
       </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/108_avtomaticheskaya_kpp_volkswagen_tiguan_5n2/photos/01.jpg|yandex_disk://коробки передач на авито/108_avtomaticheskaya_kpp_volkswagen_tiguan_5n2/photos/02.jpg|yandex_disk://коробки передач на авито/108_avtomaticheskaya_kpp_volkswagen_tiguan_5n2/photos/03.jpg|yandex_disk://коробки передач на авито/108_avtomaticheskaya_kpp_volkswagen_tiguan_5n2/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/108_avtomaticheskaya_kpp_volkswagen_tiguan_5n2/photos/01.jpg|yandex_disk://kpp_photos/108_avtomaticheskaya_kpp_volkswagen_tiguan_5n2/photos/02.jpg|yandex_disk://kpp_photos/108_avtomaticheskaya_kpp_volkswagen_tiguan_5n2/photos/03.jpg|yandex_disk://kpp_photos/108_avtomaticheskaya_kpp_volkswagen_tiguan_5n2/photos/04.jpg</t>
         </is>
       </c>
       <c r="X112" t="inlineStr">
@@ -11411,7 +11411,7 @@
       </c>
       <c r="S113" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/109_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/01.jpg|yandex_disk://коробки передач на авито/109_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/02.jpg|yandex_disk://коробки передач на авито/109_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/03.jpg|yandex_disk://коробки передач на авито/109_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/109_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/01.jpg|yandex_disk://kpp_photos/109_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/02.jpg|yandex_disk://kpp_photos/109_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/03.jpg|yandex_disk://kpp_photos/109_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/04.jpg</t>
         </is>
       </c>
       <c r="X113" t="inlineStr">
@@ -11501,7 +11501,7 @@
       </c>
       <c r="S114" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/110_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/01.jpg|yandex_disk://коробки передач на авито/110_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/02.jpg|yandex_disk://коробки передач на авито/110_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/03.jpg|yandex_disk://коробки передач на авито/110_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/110_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/01.jpg|yandex_disk://kpp_photos/110_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/02.jpg|yandex_disk://kpp_photos/110_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/03.jpg|yandex_disk://kpp_photos/110_avtomaticheskaya_kpp_volkswagen_golf_vii_5g1/photos/04.jpg</t>
         </is>
       </c>
       <c r="X114" t="inlineStr">
@@ -11591,7 +11591,7 @@
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/111_avtomaticheskaya_kpp_volkswagen_jetta_5c6/photos/01.jpg|yandex_disk://коробки передач на авито/111_avtomaticheskaya_kpp_volkswagen_jetta_5c6/photos/02.jpg|yandex_disk://коробки передач на авито/111_avtomaticheskaya_kpp_volkswagen_jetta_5c6/photos/03.jpg|yandex_disk://коробки передач на авито/111_avtomaticheskaya_kpp_volkswagen_jetta_5c6/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/111_avtomaticheskaya_kpp_volkswagen_jetta_5c6/photos/01.jpg|yandex_disk://kpp_photos/111_avtomaticheskaya_kpp_volkswagen_jetta_5c6/photos/02.jpg|yandex_disk://kpp_photos/111_avtomaticheskaya_kpp_volkswagen_jetta_5c6/photos/03.jpg|yandex_disk://kpp_photos/111_avtomaticheskaya_kpp_volkswagen_jetta_5c6/photos/04.jpg</t>
         </is>
       </c>
       <c r="X115" t="inlineStr">
@@ -11681,7 +11681,7 @@
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/112_avtomaticheskaya_kpp_volkswagen_golf_v_1k5/photos/01.jpg|yandex_disk://коробки передач на авито/112_avtomaticheskaya_kpp_volkswagen_golf_v_1k5/photos/02.jpg|yandex_disk://коробки передач на авито/112_avtomaticheskaya_kpp_volkswagen_golf_v_1k5/photos/03.jpg|yandex_disk://коробки передач на авито/112_avtomaticheskaya_kpp_volkswagen_golf_v_1k5/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/112_avtomaticheskaya_kpp_volkswagen_golf_v_1k5/photos/01.jpg|yandex_disk://kpp_photos/112_avtomaticheskaya_kpp_volkswagen_golf_v_1k5/photos/02.jpg|yandex_disk://kpp_photos/112_avtomaticheskaya_kpp_volkswagen_golf_v_1k5/photos/03.jpg|yandex_disk://kpp_photos/112_avtomaticheskaya_kpp_volkswagen_golf_v_1k5/photos/04.jpg</t>
         </is>
       </c>
       <c r="X116" t="inlineStr">
@@ -11771,7 +11771,7 @@
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/113_avtomaticheskaya_kpp_volkswagen_touran_1t2/photos/01.jpg|yandex_disk://коробки передач на авито/113_avtomaticheskaya_kpp_volkswagen_touran_1t2/photos/02.jpg|yandex_disk://коробки передач на авито/113_avtomaticheskaya_kpp_volkswagen_touran_1t2/photos/03.jpg|yandex_disk://коробки передач на авито/113_avtomaticheskaya_kpp_volkswagen_touran_1t2/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/113_avtomaticheskaya_kpp_volkswagen_touran_1t2/photos/01.jpg|yandex_disk://kpp_photos/113_avtomaticheskaya_kpp_volkswagen_touran_1t2/photos/02.jpg|yandex_disk://kpp_photos/113_avtomaticheskaya_kpp_volkswagen_touran_1t2/photos/03.jpg|yandex_disk://kpp_photos/113_avtomaticheskaya_kpp_volkswagen_touran_1t2/photos/04.jpg</t>
         </is>
       </c>
       <c r="X117" t="inlineStr">
@@ -11861,7 +11861,7 @@
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/114_mehanicheskaya_kpp_volkswagen_golf_vi_5k1/photos/01.jpg|yandex_disk://коробки передач на авито/114_mehanicheskaya_kpp_volkswagen_golf_vi_5k1/photos/02.jpg|yandex_disk://коробки передач на авито/114_mehanicheskaya_kpp_volkswagen_golf_vi_5k1/photos/03.jpg|yandex_disk://коробки передач на авито/114_mehanicheskaya_kpp_volkswagen_golf_vi_5k1/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/114_mehanicheskaya_kpp_volkswagen_golf_vi_5k1/photos/01.jpg|yandex_disk://kpp_photos/114_mehanicheskaya_kpp_volkswagen_golf_vi_5k1/photos/02.jpg|yandex_disk://kpp_photos/114_mehanicheskaya_kpp_volkswagen_golf_vi_5k1/photos/03.jpg|yandex_disk://kpp_photos/114_mehanicheskaya_kpp_volkswagen_golf_vi_5k1/photos/04.jpg</t>
         </is>
       </c>
       <c r="X118" t="inlineStr">
@@ -11951,7 +11951,7 @@
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/115_mehanicheskaya_kpp_volkswagen_polo_6r1/photos/01.jpg|yandex_disk://коробки передач на авито/115_mehanicheskaya_kpp_volkswagen_polo_6r1/photos/02.jpg|yandex_disk://коробки передач на авито/115_mehanicheskaya_kpp_volkswagen_polo_6r1/photos/03.jpg|yandex_disk://коробки передач на авито/115_mehanicheskaya_kpp_volkswagen_polo_6r1/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/115_mehanicheskaya_kpp_volkswagen_polo_6r1/photos/01.jpg|yandex_disk://kpp_photos/115_mehanicheskaya_kpp_volkswagen_polo_6r1/photos/02.jpg|yandex_disk://kpp_photos/115_mehanicheskaya_kpp_volkswagen_polo_6r1/photos/03.jpg|yandex_disk://kpp_photos/115_mehanicheskaya_kpp_volkswagen_polo_6r1/photos/04.jpg</t>
         </is>
       </c>
       <c r="X119" t="inlineStr">
@@ -12041,7 +12041,7 @@
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/116_avtomaticheskaya_kpp_volvo_v40_mv/photos/01.jpg|yandex_disk://коробки передач на авито/116_avtomaticheskaya_kpp_volvo_v40_mv/photos/02.jpg|yandex_disk://коробки передач на авито/116_avtomaticheskaya_kpp_volvo_v40_mv/photos/03.jpg|yandex_disk://коробки передач на авито/116_avtomaticheskaya_kpp_volvo_v40_mv/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/116_avtomaticheskaya_kpp_volvo_v40_mv/photos/01.jpg|yandex_disk://kpp_photos/116_avtomaticheskaya_kpp_volvo_v40_mv/photos/02.jpg|yandex_disk://kpp_photos/116_avtomaticheskaya_kpp_volvo_v40_mv/photos/03.jpg|yandex_disk://kpp_photos/116_avtomaticheskaya_kpp_volvo_v40_mv/photos/04.jpg</t>
         </is>
       </c>
       <c r="X120" t="inlineStr">
@@ -12130,7 +12130,7 @@
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>yandex_disk://коробки передач на авито/117_avtomaticheskaya_kpp_volvo_s40_vs14/photos/01.jpg|yandex_disk://коробки передач на авито/117_avtomaticheskaya_kpp_volvo_s40_vs14/photos/02.jpg|yandex_disk://коробки передач на авито/117_avtomaticheskaya_kpp_volvo_s40_vs14/photos/03.jpg|yandex_disk://коробки передач на авито/117_avtomaticheskaya_kpp_volvo_s40_vs14/photos/04.jpg</t>
+          <t>yandex_disk://kpp_photos/117_avtomaticheskaya_kpp_volvo_s40_vs14/photos/01.jpg|yandex_disk://kpp_photos/117_avtomaticheskaya_kpp_volvo_s40_vs14/photos/02.jpg|yandex_disk://kpp_photos/117_avtomaticheskaya_kpp_volvo_s40_vs14/photos/03.jpg|yandex_disk://kpp_photos/117_avtomaticheskaya_kpp_volvo_s40_vs14/photos/04.jpg</t>
         </is>
       </c>
       <c r="X121" t="inlineStr">

</xml_diff>

<commit_message>
Update kpp.xlsx: markup range widened to 9000-30000
</commit_message>
<xml_diff>
--- a/kpp.xlsx
+++ b/kpp.xlsx
@@ -1740,7 +1740,7 @@
         </is>
       </c>
       <c r="AH5" t="n">
-        <v>121500</v>
+        <v>131000</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="AH6" t="n">
-        <v>101000</v>
+        <v>108500</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
       <c r="AH7" t="n">
-        <v>101000</v>
+        <v>108500</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="AH8" t="n">
-        <v>101000</v>
+        <v>108500</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
@@ -2100,7 +2100,7 @@
         </is>
       </c>
       <c r="AH9" t="n">
-        <v>95500</v>
+        <v>103000</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="AH10" t="n">
-        <v>95500</v>
+        <v>103000</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
@@ -2280,7 +2280,7 @@
         </is>
       </c>
       <c r="AH11" t="n">
-        <v>95500</v>
+        <v>103000</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
@@ -2370,7 +2370,7 @@
         </is>
       </c>
       <c r="AH12" t="n">
-        <v>85500</v>
+        <v>92000</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
         </is>
       </c>
       <c r="AH13" t="n">
-        <v>85500</v>
+        <v>92000</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="AH14" t="n">
-        <v>85500</v>
+        <v>92000</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="AH15" t="n">
-        <v>85500</v>
+        <v>92000</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
@@ -2730,7 +2730,7 @@
         </is>
       </c>
       <c r="AH16" t="n">
-        <v>80500</v>
+        <v>86500</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="AH17" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
@@ -2909,7 +2909,7 @@
         </is>
       </c>
       <c r="AH18" t="n">
-        <v>32000</v>
+        <v>33400</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="AH19" t="n">
-        <v>31000</v>
+        <v>31800</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
@@ -3089,7 +3089,7 @@
         </is>
       </c>
       <c r="AH20" t="n">
-        <v>182500</v>
+        <v>197500</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
@@ -3179,7 +3179,7 @@
         </is>
       </c>
       <c r="AH21" t="n">
-        <v>111000</v>
+        <v>119500</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="AH22" t="n">
-        <v>101000</v>
+        <v>108500</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="AH23" t="n">
-        <v>101000</v>
+        <v>108500</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="AH24" t="n">
-        <v>101000</v>
+        <v>108500</v>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
         </is>
       </c>
       <c r="AH25" t="n">
-        <v>60000</v>
+        <v>64000</v>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="AH26" t="n">
-        <v>60000</v>
+        <v>64000</v>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
@@ -3714,7 +3714,7 @@
         </is>
       </c>
       <c r="AH27" t="n">
-        <v>55000</v>
+        <v>58500</v>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
@@ -3803,7 +3803,7 @@
         </is>
       </c>
       <c r="AH28" t="n">
-        <v>55000</v>
+        <v>58500</v>
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
@@ -3892,7 +3892,7 @@
         </is>
       </c>
       <c r="AH29" t="n">
-        <v>49500</v>
+        <v>53000</v>
       </c>
       <c r="AJ29" t="inlineStr">
         <is>
@@ -3981,7 +3981,7 @@
         </is>
       </c>
       <c r="AH30" t="n">
-        <v>44500</v>
+        <v>47500</v>
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
@@ -4070,7 +4070,7 @@
         </is>
       </c>
       <c r="AH31" t="n">
-        <v>44500</v>
+        <v>47500</v>
       </c>
       <c r="AJ31" t="inlineStr">
         <is>
@@ -4159,7 +4159,7 @@
         </is>
       </c>
       <c r="AH32" t="n">
-        <v>44500</v>
+        <v>47500</v>
       </c>
       <c r="AJ32" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="AH33" t="n">
-        <v>37500</v>
+        <v>39500</v>
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="AH34" t="n">
-        <v>90500</v>
+        <v>97500</v>
       </c>
       <c r="AJ34" t="inlineStr">
         <is>
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="AH35" t="n">
-        <v>85500</v>
+        <v>92000</v>
       </c>
       <c r="AJ35" t="inlineStr">
         <is>
@@ -4516,7 +4516,7 @@
         </is>
       </c>
       <c r="AH36" t="n">
-        <v>85500</v>
+        <v>92000</v>
       </c>
       <c r="AJ36" t="inlineStr">
         <is>
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="AH37" t="n">
-        <v>85500</v>
+        <v>92000</v>
       </c>
       <c r="AJ37" t="inlineStr">
         <is>
@@ -4695,7 +4695,7 @@
         </is>
       </c>
       <c r="AH38" t="n">
-        <v>85500</v>
+        <v>92000</v>
       </c>
       <c r="AJ38" t="inlineStr">
         <is>
@@ -4784,7 +4784,7 @@
         </is>
       </c>
       <c r="AH39" t="n">
-        <v>80500</v>
+        <v>86500</v>
       </c>
       <c r="AJ39" t="inlineStr">
         <is>
@@ -4873,7 +4873,7 @@
         </is>
       </c>
       <c r="AH40" t="n">
-        <v>80500</v>
+        <v>86500</v>
       </c>
       <c r="AJ40" t="inlineStr">
         <is>
@@ -4963,7 +4963,7 @@
         </is>
       </c>
       <c r="AH41" t="n">
-        <v>60000</v>
+        <v>64000</v>
       </c>
       <c r="AJ41" t="inlineStr">
         <is>
@@ -5053,7 +5053,7 @@
         </is>
       </c>
       <c r="AH42" t="n">
-        <v>52000</v>
+        <v>55000</v>
       </c>
       <c r="AJ42" t="inlineStr">
         <is>
@@ -5143,7 +5143,7 @@
         </is>
       </c>
       <c r="AH43" t="n">
-        <v>75500</v>
+        <v>80500</v>
       </c>
       <c r="AJ43" t="inlineStr">
         <is>
@@ -5233,7 +5233,7 @@
         </is>
       </c>
       <c r="AH44" t="n">
-        <v>157000</v>
+        <v>170000</v>
       </c>
       <c r="AJ44" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
         </is>
       </c>
       <c r="AH45" t="n">
-        <v>121500</v>
+        <v>131000</v>
       </c>
       <c r="AJ45" t="inlineStr">
         <is>
@@ -5413,7 +5413,7 @@
         </is>
       </c>
       <c r="AH46" t="n">
-        <v>95500</v>
+        <v>103000</v>
       </c>
       <c r="AJ46" t="inlineStr">
         <is>
@@ -5502,7 +5502,7 @@
         </is>
       </c>
       <c r="AH47" t="n">
-        <v>55000</v>
+        <v>58500</v>
       </c>
       <c r="AJ47" t="inlineStr">
         <is>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="AH48" t="n">
-        <v>55000</v>
+        <v>58500</v>
       </c>
       <c r="AJ48" t="inlineStr">
         <is>
@@ -5681,7 +5681,7 @@
         </is>
       </c>
       <c r="AH49" t="n">
-        <v>29500</v>
+        <v>30500</v>
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
@@ -5771,7 +5771,7 @@
         </is>
       </c>
       <c r="AH50" t="n">
-        <v>203000</v>
+        <v>220000</v>
       </c>
       <c r="AJ50" t="inlineStr">
         <is>
@@ -5861,7 +5861,7 @@
         </is>
       </c>
       <c r="AH51" t="n">
-        <v>198000</v>
+        <v>214500</v>
       </c>
       <c r="AJ51" t="inlineStr">
         <is>
@@ -5951,7 +5951,7 @@
         </is>
       </c>
       <c r="AH52" t="n">
-        <v>141500</v>
+        <v>153000</v>
       </c>
       <c r="AJ52" t="inlineStr">
         <is>
@@ -6040,7 +6040,7 @@
         </is>
       </c>
       <c r="AH53" t="n">
-        <v>111000</v>
+        <v>119500</v>
       </c>
       <c r="AJ53" t="inlineStr">
         <is>
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="AH54" t="n">
-        <v>49500</v>
+        <v>53000</v>
       </c>
       <c r="AJ54" t="inlineStr">
         <is>
@@ -6218,7 +6218,7 @@
         </is>
       </c>
       <c r="AH55" t="n">
-        <v>36500</v>
+        <v>38500</v>
       </c>
       <c r="AJ55" t="inlineStr">
         <is>
@@ -6308,7 +6308,7 @@
         </is>
       </c>
       <c r="AH56" t="n">
-        <v>101000</v>
+        <v>108500</v>
       </c>
       <c r="AJ56" t="inlineStr">
         <is>
@@ -6397,7 +6397,7 @@
         </is>
       </c>
       <c r="AH57" t="n">
-        <v>65000</v>
+        <v>69500</v>
       </c>
       <c r="AJ57" t="inlineStr">
         <is>
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="AH58" t="n">
-        <v>106000</v>
+        <v>114000</v>
       </c>
       <c r="AJ58" t="inlineStr">
         <is>
@@ -6576,7 +6576,7 @@
         </is>
       </c>
       <c r="AH59" t="n">
-        <v>49500</v>
+        <v>53000</v>
       </c>
       <c r="AJ59" t="inlineStr">
         <is>
@@ -6666,7 +6666,7 @@
         </is>
       </c>
       <c r="AH60" t="n">
-        <v>19000</v>
+        <v>19500</v>
       </c>
       <c r="AJ60" t="inlineStr">
         <is>
@@ -6756,7 +6756,7 @@
         </is>
       </c>
       <c r="AH61" t="n">
-        <v>44500</v>
+        <v>47500</v>
       </c>
       <c r="AJ61" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         </is>
       </c>
       <c r="AH62" t="n">
-        <v>44500</v>
+        <v>47500</v>
       </c>
       <c r="AJ62" t="inlineStr">
         <is>
@@ -6935,7 +6935,7 @@
         </is>
       </c>
       <c r="AH63" t="n">
-        <v>36500</v>
+        <v>38500</v>
       </c>
       <c r="AJ63" t="inlineStr">
         <is>
@@ -7025,7 +7025,7 @@
         </is>
       </c>
       <c r="AH64" t="n">
-        <v>34500</v>
+        <v>36000</v>
       </c>
       <c r="AJ64" t="inlineStr">
         <is>
@@ -7115,7 +7115,7 @@
         </is>
       </c>
       <c r="AH65" t="n">
-        <v>31500</v>
+        <v>33000</v>
       </c>
       <c r="AJ65" t="inlineStr">
         <is>
@@ -7205,7 +7205,7 @@
         </is>
       </c>
       <c r="AH66" t="n">
-        <v>31500</v>
+        <v>33000</v>
       </c>
       <c r="AJ66" t="inlineStr">
         <is>
@@ -7294,7 +7294,7 @@
         </is>
       </c>
       <c r="AH67" t="n">
-        <v>27500</v>
+        <v>28500</v>
       </c>
       <c r="AJ67" t="inlineStr">
         <is>
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="AH68" t="n">
-        <v>18000</v>
+        <v>18500</v>
       </c>
       <c r="AJ68" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
         </is>
       </c>
       <c r="AH69" t="n">
-        <v>18000</v>
+        <v>18500</v>
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
@@ -7563,7 +7563,7 @@
         </is>
       </c>
       <c r="AH70" t="n">
-        <v>75500</v>
+        <v>80500</v>
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
@@ -7652,7 +7652,7 @@
         </is>
       </c>
       <c r="AH71" t="n">
-        <v>44500</v>
+        <v>47500</v>
       </c>
       <c r="AJ71" t="inlineStr">
         <is>
@@ -7742,7 +7742,7 @@
         </is>
       </c>
       <c r="AH72" t="n">
-        <v>21000</v>
+        <v>21500</v>
       </c>
       <c r="AJ72" t="inlineStr">
         <is>
@@ -7831,7 +7831,7 @@
         </is>
       </c>
       <c r="AH73" t="n">
-        <v>75500</v>
+        <v>80500</v>
       </c>
       <c r="AJ73" t="inlineStr">
         <is>
@@ -7921,7 +7921,7 @@
         </is>
       </c>
       <c r="AH74" t="n">
-        <v>49500</v>
+        <v>53000</v>
       </c>
       <c r="AJ74" t="inlineStr">
         <is>
@@ -8011,7 +8011,7 @@
         </is>
       </c>
       <c r="AH75" t="n">
-        <v>32000</v>
+        <v>33400</v>
       </c>
       <c r="AJ75" t="inlineStr">
         <is>
@@ -8101,7 +8101,7 @@
         </is>
       </c>
       <c r="AH76" t="n">
-        <v>111000</v>
+        <v>119500</v>
       </c>
       <c r="AJ76" t="inlineStr">
         <is>
@@ -8191,7 +8191,7 @@
         </is>
       </c>
       <c r="AH77" t="n">
-        <v>95500</v>
+        <v>103000</v>
       </c>
       <c r="AJ77" t="inlineStr">
         <is>
@@ -8281,7 +8281,7 @@
         </is>
       </c>
       <c r="AH78" t="n">
-        <v>53000</v>
+        <v>56000</v>
       </c>
       <c r="AJ78" t="inlineStr">
         <is>
@@ -8371,7 +8371,7 @@
         </is>
       </c>
       <c r="AH79" t="n">
-        <v>49500</v>
+        <v>53000</v>
       </c>
       <c r="AJ79" t="inlineStr">
         <is>
@@ -8461,7 +8461,7 @@
         </is>
       </c>
       <c r="AH80" t="n">
-        <v>49500</v>
+        <v>53000</v>
       </c>
       <c r="AJ80" t="inlineStr">
         <is>
@@ -8551,7 +8551,7 @@
         </is>
       </c>
       <c r="AH81" t="n">
-        <v>44500</v>
+        <v>47500</v>
       </c>
       <c r="AJ81" t="inlineStr">
         <is>
@@ -8641,7 +8641,7 @@
         </is>
       </c>
       <c r="AH82" t="n">
-        <v>39500</v>
+        <v>41500</v>
       </c>
       <c r="AJ82" t="inlineStr">
         <is>
@@ -8731,7 +8731,7 @@
         </is>
       </c>
       <c r="AH83" t="n">
-        <v>126500</v>
+        <v>136500</v>
       </c>
       <c r="AJ83" t="inlineStr">
         <is>
@@ -8821,7 +8821,7 @@
         </is>
       </c>
       <c r="AH84" t="n">
-        <v>121500</v>
+        <v>131000</v>
       </c>
       <c r="AJ84" t="inlineStr">
         <is>
@@ -8911,7 +8911,7 @@
         </is>
       </c>
       <c r="AH85" t="n">
-        <v>111000</v>
+        <v>119500</v>
       </c>
       <c r="AJ85" t="inlineStr">
         <is>
@@ -9000,7 +9000,7 @@
         </is>
       </c>
       <c r="AH86" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
       <c r="AJ86" t="inlineStr">
         <is>
@@ -9090,7 +9090,7 @@
         </is>
       </c>
       <c r="AH87" t="n">
-        <v>95500</v>
+        <v>103000</v>
       </c>
       <c r="AJ87" t="inlineStr">
         <is>
@@ -9180,7 +9180,7 @@
         </is>
       </c>
       <c r="AH88" t="n">
-        <v>63000</v>
+        <v>67500</v>
       </c>
       <c r="AJ88" t="inlineStr">
         <is>
@@ -9270,7 +9270,7 @@
         </is>
       </c>
       <c r="AH89" t="n">
-        <v>32000</v>
+        <v>33400</v>
       </c>
       <c r="AJ89" t="inlineStr">
         <is>
@@ -9360,7 +9360,7 @@
         </is>
       </c>
       <c r="AH90" t="n">
-        <v>26000</v>
+        <v>26800</v>
       </c>
       <c r="AJ90" t="inlineStr">
         <is>
@@ -9449,7 +9449,7 @@
         </is>
       </c>
       <c r="AH91" t="n">
-        <v>24000</v>
+        <v>25000</v>
       </c>
       <c r="AJ91" t="inlineStr">
         <is>
@@ -9539,7 +9539,7 @@
         </is>
       </c>
       <c r="AH92" t="n">
-        <v>29500</v>
+        <v>30500</v>
       </c>
       <c r="AJ92" t="inlineStr">
         <is>
@@ -9629,7 +9629,7 @@
         </is>
       </c>
       <c r="AH93" t="n">
-        <v>101000</v>
+        <v>108500</v>
       </c>
       <c r="AJ93" t="inlineStr">
         <is>
@@ -9718,7 +9718,7 @@
         </is>
       </c>
       <c r="AH94" t="n">
-        <v>80500</v>
+        <v>86500</v>
       </c>
       <c r="AJ94" t="inlineStr">
         <is>
@@ -9808,7 +9808,7 @@
         </is>
       </c>
       <c r="AH95" t="n">
-        <v>44500</v>
+        <v>47500</v>
       </c>
       <c r="AJ95" t="inlineStr">
         <is>
@@ -9898,7 +9898,7 @@
         </is>
       </c>
       <c r="AH96" t="n">
-        <v>39500</v>
+        <v>41500</v>
       </c>
       <c r="AJ96" t="inlineStr">
         <is>
@@ -9987,7 +9987,7 @@
         </is>
       </c>
       <c r="AH97" t="n">
-        <v>34500</v>
+        <v>36000</v>
       </c>
       <c r="AJ97" t="inlineStr">
         <is>
@@ -10076,7 +10076,7 @@
         </is>
       </c>
       <c r="AH98" t="n">
-        <v>59500</v>
+        <v>63500</v>
       </c>
       <c r="AJ98" t="inlineStr">
         <is>
@@ -10166,7 +10166,7 @@
         </is>
       </c>
       <c r="AH99" t="n">
-        <v>80500</v>
+        <v>86500</v>
       </c>
       <c r="AJ99" t="inlineStr">
         <is>
@@ -10256,7 +10256,7 @@
         </is>
       </c>
       <c r="AH100" t="n">
-        <v>70000</v>
+        <v>75000</v>
       </c>
       <c r="AJ100" t="inlineStr">
         <is>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="AH102" t="n">
-        <v>43000</v>
+        <v>45600</v>
       </c>
       <c r="AJ102" t="inlineStr">
         <is>
@@ -10525,7 +10525,7 @@
         </is>
       </c>
       <c r="AH103" t="n">
-        <v>121500</v>
+        <v>131000</v>
       </c>
       <c r="AJ103" t="inlineStr">
         <is>
@@ -10614,7 +10614,7 @@
         </is>
       </c>
       <c r="AH104" t="n">
-        <v>121500</v>
+        <v>131000</v>
       </c>
       <c r="AJ104" t="inlineStr">
         <is>
@@ -10704,7 +10704,7 @@
         </is>
       </c>
       <c r="AH105" t="n">
-        <v>111000</v>
+        <v>119500</v>
       </c>
       <c r="AJ105" t="inlineStr">
         <is>
@@ -10793,7 +10793,7 @@
         </is>
       </c>
       <c r="AH106" t="n">
-        <v>101000</v>
+        <v>108500</v>
       </c>
       <c r="AJ106" t="inlineStr">
         <is>
@@ -10882,7 +10882,7 @@
         </is>
       </c>
       <c r="AH107" t="n">
-        <v>95500</v>
+        <v>103000</v>
       </c>
       <c r="AJ107" t="inlineStr">
         <is>
@@ -10971,7 +10971,7 @@
         </is>
       </c>
       <c r="AH108" t="n">
-        <v>39500</v>
+        <v>41500</v>
       </c>
       <c r="AJ108" t="inlineStr">
         <is>
@@ -11061,7 +11061,7 @@
         </is>
       </c>
       <c r="AH109" t="n">
-        <v>21000</v>
+        <v>21500</v>
       </c>
       <c r="AJ109" t="inlineStr">
         <is>
@@ -11150,7 +11150,7 @@
         </is>
       </c>
       <c r="AH110" t="n">
-        <v>40000</v>
+        <v>42300</v>
       </c>
       <c r="AJ110" t="inlineStr">
         <is>
@@ -11240,7 +11240,7 @@
         </is>
       </c>
       <c r="AH111" t="n">
-        <v>172500</v>
+        <v>186500</v>
       </c>
       <c r="AJ111" t="inlineStr">
         <is>
@@ -11330,7 +11330,7 @@
         </is>
       </c>
       <c r="AH112" t="n">
-        <v>136500</v>
+        <v>147500</v>
       </c>
       <c r="AJ112" t="inlineStr">
         <is>
@@ -11420,7 +11420,7 @@
         </is>
       </c>
       <c r="AH113" t="n">
-        <v>90500</v>
+        <v>97500</v>
       </c>
       <c r="AJ113" t="inlineStr">
         <is>
@@ -11510,7 +11510,7 @@
         </is>
       </c>
       <c r="AH114" t="n">
-        <v>90500</v>
+        <v>97500</v>
       </c>
       <c r="AJ114" t="inlineStr">
         <is>
@@ -11600,7 +11600,7 @@
         </is>
       </c>
       <c r="AH115" t="n">
-        <v>80500</v>
+        <v>86500</v>
       </c>
       <c r="AJ115" t="inlineStr">
         <is>
@@ -11690,7 +11690,7 @@
         </is>
       </c>
       <c r="AH116" t="n">
-        <v>60000</v>
+        <v>64000</v>
       </c>
       <c r="AJ116" t="inlineStr">
         <is>
@@ -11780,7 +11780,7 @@
         </is>
       </c>
       <c r="AH117" t="n">
-        <v>55000</v>
+        <v>58500</v>
       </c>
       <c r="AJ117" t="inlineStr">
         <is>
@@ -11870,7 +11870,7 @@
         </is>
       </c>
       <c r="AH118" t="n">
-        <v>70500</v>
+        <v>75500</v>
       </c>
       <c r="AJ118" t="inlineStr">
         <is>
@@ -11960,7 +11960,7 @@
         </is>
       </c>
       <c r="AH119" t="n">
-        <v>55000</v>
+        <v>58500</v>
       </c>
       <c r="AJ119" t="inlineStr">
         <is>
@@ -12050,7 +12050,7 @@
         </is>
       </c>
       <c r="AH120" t="n">
-        <v>34500</v>
+        <v>36000</v>
       </c>
       <c r="AJ120" t="inlineStr">
         <is>
@@ -12139,7 +12139,7 @@
         </is>
       </c>
       <c r="AH121" t="n">
-        <v>29500</v>
+        <v>30500</v>
       </c>
       <c r="AJ121" t="inlineStr">
         <is>

</xml_diff>